<commit_message>
"Relation: Source Object Var Name" column in Db Column definition removed (not needed)
</commit_message>
<xml_diff>
--- a/excel-format/db-column-definitions_fmt-v5.0.0-en_my-app.xlsx
+++ b/excel-format/db-column-definitions_fmt-v5.0.0-en_my-app.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yosuke.tanaka/Desktop/development/git/ecuacion-tool-code-generator/excel-format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F46F3CBA-1473-4246-9034-2C7E81A23414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B6E3358-FD95-8040-8650-CF7A3F8B8688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="11700" tabRatio="853" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="11700" tabRatio="853" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="dataType Dropdown Items" sheetId="1" state="hidden" r:id="rId1"/>
@@ -29,7 +29,7 @@
   </externalReferences>
   <definedNames>
     <definedName name="general">'dataType Dropdown Items'!$A$3:$A$18</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="7">'DB Item Definition'!$A$1:$Z$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="7">'DB Item Definition'!$A$1:$Y$5</definedName>
     <definedName name="一般">[1]dataTypeプルダウン項目!$A$3:$A$16</definedName>
     <definedName name="固定フォーマット">[1]dataTypeプルダウン項目!#REF!</definedName>
     <definedName name="日時">[1]dataTypeプルダウン項目!#REF!</definedName>
@@ -128,7 +128,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="215">
   <si>
     <t>DB Common Item Definition</t>
   </si>
@@ -194,9 +194,6 @@
   </si>
   <si>
     <t>Relation: Source Var Name</t>
-  </si>
-  <si>
-    <t>Relation: Source Object Var Name</t>
   </si>
   <si>
     <t>Relation: Target Table</t>
@@ -1570,7 +1567,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="標準 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
-  <dxfs count="125">
+  <dxfs count="123">
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="center"/>
@@ -1970,22 +1967,6 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="center" vertical="center"/>
-      <border>
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -2521,11 +2502,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
@@ -3092,113 +3068,113 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table5" displayName="Table5" ref="A3:D4" totalsRowShown="0" headerRowDxfId="115" dataDxfId="114">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table5" displayName="Table5" ref="A3:D4" totalsRowShown="0" headerRowDxfId="113" dataDxfId="112">
   <autoFilter ref="A3:D4" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Date" dataDxfId="113"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Version" dataDxfId="112"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Changes" dataDxfId="111"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Changed By" dataDxfId="110"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Date" dataDxfId="111"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Version" dataDxfId="110"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Changes" dataDxfId="109"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Changed By" dataDxfId="108"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table50" displayName="Table50" ref="A5:H28" totalsRowShown="0" dataDxfId="124">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table50" displayName="Table50" ref="A5:H28" totalsRowShown="0" dataDxfId="122">
   <autoFilter ref="A5:H28" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="#" dataDxfId="123">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="#" dataDxfId="121">
       <calculatedColumnFormula>ROW()-5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="Category" dataDxfId="122"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Category Name" dataDxfId="121"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Key" dataDxfId="120"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Description" dataDxfId="119"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="Required" dataDxfId="118"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Value" dataDxfId="117"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Notes" dataDxfId="116"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="Category" dataDxfId="120"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Category Name" dataDxfId="119"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Key" dataDxfId="118"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Description" dataDxfId="117"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="Required" dataDxfId="116"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Value" dataDxfId="115"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Notes" dataDxfId="114"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table2" displayName="Table2" ref="A7:S45" tableType="xml" totalsRowShown="0" headerRowDxfId="109" dataDxfId="108">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table2" displayName="Table2" ref="A7:S45" tableType="xml" totalsRowShown="0" headerRowDxfId="107" dataDxfId="106">
   <tableColumns count="19">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" uniqueName="name" name="DataType Name" dataDxfId="107">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" uniqueName="name" name="DataType Name" dataDxfId="105">
       <xmlColumnPr mapId="191" xpath="/root/datatype/@name" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" uniqueName="kata" name="Type" dataDxfId="106">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" uniqueName="kata" name="Type" dataDxfId="104">
       <xmlColumnPr mapId="191" xpath="/root/datatype/kata" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" uniqueName="minLength" name="Min Length" dataDxfId="105">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" uniqueName="minLength" name="Min Length" dataDxfId="103">
       <xmlColumnPr mapId="191" xpath="/root/datatype/minLength" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0400-00000B000000}" uniqueName="maxLength" name="Max Length" dataDxfId="104">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0400-00000B000000}" uniqueName="maxLength" name="Max Length" dataDxfId="102">
       <xmlColumnPr mapId="191" xpath="/root/datatype/maxLength" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0400-00000F000000}" uniqueName="numScale" name="Data Pattern (display name)" dataDxfId="103"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0400-000018000000}" uniqueName="stringDataPtn" name="Data Pattern" dataDxfId="102">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0400-00000F000000}" uniqueName="numScale" name="Data Pattern (display name)" dataDxfId="101"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0400-000018000000}" uniqueName="stringDataPtn" name="Data Pattern" dataDxfId="100">
       <xmlColumnPr mapId="191" xpath="/root/datatype/stringDataPtn" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0400-000012000000}" uniqueName="18" name="Exclude Prohibited Chars Check" dataDxfId="101"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0400-000019000000}" uniqueName="stringRegEx" name="Regex" dataDxfId="100">
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0400-000012000000}" uniqueName="18" name="Exclude Prohibited Chars Check" dataDxfId="99"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0400-000019000000}" uniqueName="stringRegEx" name="Regex" dataDxfId="98">
       <xmlColumnPr mapId="191" xpath="/root/datatype/stringRegEx" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" uniqueName="numMinVal" name="Min Value" dataDxfId="99">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" uniqueName="numMinVal" name="Min Value" dataDxfId="97">
       <xmlColumnPr mapId="191" xpath="/root/datatype/numMinVal" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0400-00000A000000}" uniqueName="numMaxVal" name="Max Value" dataDxfId="98">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0400-00000A000000}" uniqueName="numMaxVal" name="Max Value" dataDxfId="96">
       <xmlColumnPr mapId="191" xpath="/root/datatype/numMaxVal" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0400-00000C000000}" uniqueName="numDigitInteger" name="Integer Digits" dataDxfId="97">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0400-00000C000000}" uniqueName="numDigitInteger" name="Integer Digits" dataDxfId="95">
       <xmlColumnPr mapId="191" xpath="/root/datatype/numDigitInteger" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0400-00000D000000}" uniqueName="numDigitFraction" name="Decimal Digits" dataDxfId="96">
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0400-00000D000000}" uniqueName="numDigitFraction" name="Decimal Digits" dataDxfId="94">
       <xmlColumnPr mapId="191" xpath="/root/datatype/numDigitFraction" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" uniqueName="enumCodeLength" name="Code Length" dataDxfId="95">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" uniqueName="enumCodeLength" name="Code Length" dataDxfId="93">
       <xmlColumnPr mapId="191" xpath="/root/datatype/enumCodeLength" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0400-00000E000000}" uniqueName="notNeedsTimezone" name="No Timezone" dataDxfId="94">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0400-00000E000000}" uniqueName="notNeedsTimezone" name="No Timezone" dataDxfId="92">
       <xmlColumnPr mapId="191" xpath="/root/datatype/notNeedsTimezone" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0400-000010000000}" uniqueName="javadoc" name="Notes" dataDxfId="93">
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0400-000010000000}" uniqueName="javadoc" name="Notes" dataDxfId="91">
       <xmlColumnPr mapId="191" xpath="/root/datatype/javadoc" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" uniqueName="2" name="Pattern Desc (Default Lang)" dataDxfId="92"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0400-000013000000}" uniqueName="19" name="Pattern Desc (Additional Lang 1)" dataDxfId="91"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0400-000014000000}" uniqueName="20" name="Pattern Desc (Additional Lang 2)" dataDxfId="90"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0400-000015000000}" uniqueName="21" name="Pattern Desc (Additional Lang 3)" dataDxfId="89"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" uniqueName="2" name="Pattern Desc (Default Lang)" dataDxfId="90"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0400-000013000000}" uniqueName="19" name="Pattern Desc (Additional Lang 1)" dataDxfId="89"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0400-000014000000}" uniqueName="20" name="Pattern Desc (Additional Lang 2)" dataDxfId="88"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0400-000015000000}" uniqueName="21" name="Pattern Desc (Additional Lang 3)" dataDxfId="87"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Table4" displayName="Table4" ref="A6:I33" tableType="xml" totalsRowShown="0" headerRowDxfId="88" dataDxfId="87">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Table4" displayName="Table4" ref="A6:I33" tableType="xml" totalsRowShown="0" headerRowDxfId="86" dataDxfId="85">
   <autoFilter ref="A6:I33" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" uniqueName="dataTypeName" name="DataType Name" dataDxfId="86">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" uniqueName="dataTypeName" name="DataType Name" dataDxfId="84">
       <xmlColumnPr mapId="132" xpath="/root/enum/dataTypeName" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" uniqueName="8" name="code" dataDxfId="85"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" uniqueName="varName" name="varName" dataDxfId="84">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" uniqueName="8" name="code" dataDxfId="83"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" uniqueName="varName" name="varName" dataDxfId="82">
       <xmlColumnPr mapId="132" xpath="/root/enum/varName" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0500-00000A000000}" uniqueName="10" name="Java Only" dataDxfId="83"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0500-00000C000000}" uniqueName="javadoc-value" name="Notes" dataDxfId="82">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0500-00000A000000}" uniqueName="10" name="Java Only" dataDxfId="81"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0500-00000C000000}" uniqueName="javadoc-value" name="Notes" dataDxfId="80">
       <xmlColumnPr mapId="132" xpath="/root/enum/javadoc-value" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" uniqueName="9" name="Display Name (Default Lang)" dataDxfId="81"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" uniqueName="dispNameAddLang1" name="Display Name (Additional Lang 1)" dataDxfId="80">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" uniqueName="9" name="Display Name (Default Lang)" dataDxfId="79"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" uniqueName="dispNameAddLang1" name="Display Name (Additional Lang 1)" dataDxfId="78">
       <xmlColumnPr mapId="132" xpath="/root/enum/dispNameAddLang1" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" uniqueName="dispNameAddLang2" name="Display Name (Additional Lang 2)" dataDxfId="79">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" uniqueName="dispNameAddLang2" name="Display Name (Additional Lang 2)" dataDxfId="77">
       <xmlColumnPr mapId="132" xpath="/root/enum/dispNameAddLang2" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" uniqueName="dispNameAddLang3" name="Display Name (Additional Lang 3)" dataDxfId="78">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" uniqueName="dispNameAddLang3" name="Display Name (Additional Lang 3)" dataDxfId="76">
       <xmlColumnPr mapId="132" xpath="/root/enum/dispNameAddLang3" xmlDataType="string"/>
     </tableColumn>
   </tableColumns>
@@ -3207,82 +3183,81 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="Table7" displayName="Table7" ref="A5:AK90" tableType="xml" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
-  <autoFilter ref="A5:AK90" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
-  <tableColumns count="37">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" uniqueName="table" name="Table Name" dataDxfId="75">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="Table7" displayName="Table7" ref="A5:AJ90" tableType="xml" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
+  <autoFilter ref="A5:AJ90" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
+  <tableColumns count="36">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" uniqueName="table" name="Table Name" dataDxfId="73">
       <xmlColumnPr mapId="161" xpath="/root/column/table" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" uniqueName="name" name="Column Name" dataDxfId="74">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" uniqueName="name" name="Column Name" dataDxfId="72">
       <xmlColumnPr mapId="161" xpath="/root/column/@name" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0600-00000F000000}" uniqueName="dataType" name="dataType" dataDxfId="73">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0600-00000F000000}" uniqueName="dataType" name="dataType" dataDxfId="71">
       <xmlColumnPr mapId="161" xpath="/root/column/dataType" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0600-000010000000}" uniqueName="16" name="dataType Check" dataDxfId="72">
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0600-000010000000}" uniqueName="16" name="dataType Check" dataDxfId="70">
       <calculatedColumnFormula>IF(Table7[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table7[[#This Row],[dataType]], 'dataType Definition'!A:A, 1,FALSE))), "○", "×"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0600-00001C000000}" uniqueName="28" name="Java Only" dataDxfId="71"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" uniqueName="pk" name="Surrogate key " dataDxfId="70">
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0600-00001C000000}" uniqueName="28" name="Java Only" dataDxfId="69"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" uniqueName="pk" name="Surrogate key " dataDxfId="68">
       <xmlColumnPr mapId="161" xpath="/root/column/pk" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0600-00001D000000}" uniqueName="29" name="natural key (unique key)" dataDxfId="69"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0600-000008000000}" uniqueName="nullable" name="nullable" dataDxfId="68">
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0600-00001D000000}" uniqueName="29" name="natural key (unique key)" dataDxfId="67"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0600-000008000000}" uniqueName="nullable" name="nullable" dataDxfId="66">
       <xmlColumnPr mapId="161" xpath="/root/column/nullable" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0600-00000A000000}" uniqueName="autoIncrement" name="Auto Numbering" dataDxfId="67">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0600-00000A000000}" uniqueName="autoIncrement" name="Auto Numbering" dataDxfId="65">
       <xmlColumnPr mapId="161" xpath="/root/column/autoIncrement" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0600-000015000000}" uniqueName="forcedIncrement" name="Force Numbering" dataDxfId="66">
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0600-000015000000}" uniqueName="forcedIncrement" name="Force Numbering" dataDxfId="64">
       <xmlColumnPr mapId="161" xpath="/root/column/forcedIncrement" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0600-00000B000000}" uniqueName="autoUpdate" name="Auto Update" dataDxfId="65">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0600-00000B000000}" uniqueName="autoUpdate" name="Auto Update" dataDxfId="63">
       <xmlColumnPr mapId="161" xpath="/root/column/autoUpdate" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0600-000014000000}" uniqueName="forcedUpdate" name="Force Update" dataDxfId="64">
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0600-000014000000}" uniqueName="forcedUpdate" name="Force Update" dataDxfId="62">
       <xmlColumnPr mapId="161" xpath="/root/column/forcedUpdate" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0600-00000C000000}" uniqueName="valueChangeMethod" name="Group Identifier" dataDxfId="63">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0600-00000C000000}" uniqueName="valueChangeMethod" name="Group Identifier" dataDxfId="61">
       <xmlColumnPr mapId="161" xpath="/root/column/valueChangeMethod" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0600-000012000000}" uniqueName="updatedValue" name="Spring Audit" dataDxfId="62">
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0600-000012000000}" uniqueName="updatedValue" name="Spring Audit" dataDxfId="60">
       <xmlColumnPr mapId="161" xpath="/root/column/updatedValue" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0600-000013000000}" uniqueName="optLock" name="Relation: Type" dataDxfId="61">
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0600-000013000000}" uniqueName="optLock" name="Relation: Type" dataDxfId="59">
       <xmlColumnPr mapId="161" xpath="/root/column/optLock" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0600-000016000000}" uniqueName="22" name="Relation: Direction" dataDxfId="60"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0600-00001A000000}" uniqueName="26" name="Relation: Source Var Name" dataDxfId="59"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0600-00001E000000}" uniqueName="30" name="Relation: Source Object Var Name" dataDxfId="58"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0600-000017000000}" uniqueName="23" name="Relation: Target Table" dataDxfId="57"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0600-000018000000}" uniqueName="24" name="Relation: Target Column" dataDxfId="56"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0600-00001B000000}" uniqueName="27" name="Relation: Target Var Name" dataDxfId="55"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0600-000019000000}" uniqueName="25" name="Relation: Eager" dataDxfId="54"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0600-000011000000}" uniqueName="index1" name="index1" dataDxfId="53">
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0600-000016000000}" uniqueName="22" name="Relation: Direction" dataDxfId="58"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0600-00001A000000}" uniqueName="26" name="Relation: Source Var Name" dataDxfId="57"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0600-000017000000}" uniqueName="23" name="Relation: Target Table" dataDxfId="56"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0600-000018000000}" uniqueName="24" name="Relation: Target Column" dataDxfId="55"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0600-00001B000000}" uniqueName="27" name="Relation: Target Var Name" dataDxfId="54"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0600-000019000000}" uniqueName="25" name="Relation: Eager" dataDxfId="53"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0600-000011000000}" uniqueName="index1" name="index1" dataDxfId="52">
       <xmlColumnPr mapId="161" xpath="/root/column/index1" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0600-00000E000000}" uniqueName="index2" name="index2" dataDxfId="52">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0600-00000E000000}" uniqueName="index2" name="index2" dataDxfId="51">
       <xmlColumnPr mapId="161" xpath="/root/column/index2" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0600-00000D000000}" uniqueName="index3" name="index3" dataDxfId="51">
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0600-00000D000000}" uniqueName="index3" name="index3" dataDxfId="50">
       <xmlColumnPr mapId="161" xpath="/root/column/index3" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0600-000022000000}" uniqueName="34" name="index4" dataDxfId="50"/>
-    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0600-000023000000}" uniqueName="35" name="index5" dataDxfId="49"/>
-    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0600-000024000000}" uniqueName="36" name="index6" dataDxfId="48"/>
-    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0600-000025000000}" uniqueName="37" name="index7" dataDxfId="47"/>
-    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0600-000026000000}" uniqueName="38" name="index8" dataDxfId="46"/>
-    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0600-000027000000}" uniqueName="39" name="index9" dataDxfId="45"/>
-    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0600-000028000000}" uniqueName="40" name="index10" dataDxfId="44"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" uniqueName="dispNameAddLang1" name="Notes" dataDxfId="43"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0600-000009000000}" uniqueName="9" name="Column Display Name (Default Lang)" dataDxfId="42"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" uniqueName="dispNameAddLang1" name="Column Display Name (Additional Lang 1)" dataDxfId="41">
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0600-000022000000}" uniqueName="34" name="index4" dataDxfId="49"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0600-000023000000}" uniqueName="35" name="index5" dataDxfId="48"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0600-000024000000}" uniqueName="36" name="index6" dataDxfId="47"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0600-000025000000}" uniqueName="37" name="index7" dataDxfId="46"/>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0600-000026000000}" uniqueName="38" name="index8" dataDxfId="45"/>
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0600-000027000000}" uniqueName="39" name="index9" dataDxfId="44"/>
+    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0600-000028000000}" uniqueName="40" name="index10" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" uniqueName="dispNameAddLang1" name="Notes" dataDxfId="42"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0600-000009000000}" uniqueName="9" name="Column Display Name (Default Lang)" dataDxfId="41"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" uniqueName="dispNameAddLang1" name="Column Display Name (Additional Lang 1)" dataDxfId="40">
       <xmlColumnPr mapId="161" xpath="/root/column/dispNameAddLang1" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" uniqueName="dispNameAddLang2" name="Column Display Name (Additional Lang 2)" dataDxfId="40">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" uniqueName="dispNameAddLang2" name="Column Display Name (Additional Lang 2)" dataDxfId="39">
       <xmlColumnPr mapId="161" xpath="/root/column/dispNameAddLang2" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" uniqueName="dispNameAddLang3" name="Column Display Name (Additional Lang 3)" dataDxfId="39">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" uniqueName="dispNameAddLang3" name="Column Display Name (Additional Lang 3)" dataDxfId="38">
       <xmlColumnPr mapId="161" xpath="/root/column/dispNameAddLang3" xmlDataType="string"/>
     </tableColumn>
   </tableColumns>
@@ -3291,29 +3266,28 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="Table74" displayName="Table74" ref="A5:AK13" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
-  <autoFilter ref="A5:AK13" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
-  <tableColumns count="37">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="Table Name" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Column Name" dataDxfId="35"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0700-00000F000000}" name="dataType" dataDxfId="34"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0700-000010000000}" name="dataType Check" dataDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="Table74" displayName="Table74" ref="A5:AJ13" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
+  <autoFilter ref="A5:AJ13" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
+  <tableColumns count="36">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="Table Name" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Column Name" dataDxfId="34"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0700-00000F000000}" name="dataType" dataDxfId="33"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0700-000010000000}" name="dataType Check" dataDxfId="32">
       <calculatedColumnFormula>IF(Table74[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table74[[#This Row],[dataType]], 'dataType Definition'!A:A, 1,FALSE))), "○", "×"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0700-00001C000000}" name="Java Only" dataDxfId="32"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="Surrogate key " dataDxfId="31"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="natural key (unique key)" dataDxfId="30"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0700-00001D000000}" name="nullable" dataDxfId="29"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0700-00000A000000}" name="Auto Numbering" dataDxfId="28"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0700-000015000000}" name="Force Numbering" dataDxfId="27"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Auto Update" dataDxfId="26"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0700-000014000000}" name="Force Update" dataDxfId="25"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0700-00000C000000}" name="Group Identifier" dataDxfId="24"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0700-000012000000}" name="Spring Audit" dataDxfId="23"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0700-000013000000}" name="Relation: Type" dataDxfId="22"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0700-000016000000}" name="Relation: Direction" dataDxfId="21"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0700-00001A000000}" name="Relation: Source Var Name" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="Relation: Source Object Var Name" dataDxfId="19"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0700-00001C000000}" name="Java Only" dataDxfId="31"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="Surrogate key " dataDxfId="30"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="natural key (unique key)" dataDxfId="29"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0700-00001D000000}" name="nullable" dataDxfId="28"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0700-00000A000000}" name="Auto Numbering" dataDxfId="27"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0700-000015000000}" name="Force Numbering" dataDxfId="26"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Auto Update" dataDxfId="25"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0700-000014000000}" name="Force Update" dataDxfId="24"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0700-00000C000000}" name="Group Identifier" dataDxfId="23"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0700-000012000000}" name="Spring Audit" dataDxfId="22"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0700-000013000000}" name="Relation: Type" dataDxfId="21"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0700-000016000000}" name="Relation: Direction" dataDxfId="20"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0700-00001A000000}" name="Relation: Source Var Name" dataDxfId="19"/>
     <tableColumn id="23" xr3:uid="{00000000-0010-0000-0700-000017000000}" name="Relation: Target Table" dataDxfId="18"/>
     <tableColumn id="24" xr3:uid="{00000000-0010-0000-0700-000018000000}" name="Relation: Target Column" dataDxfId="17"/>
     <tableColumn id="27" xr3:uid="{00000000-0010-0000-0700-00001B000000}" name="Relation: Target Var Name" dataDxfId="16"/>
@@ -3635,154 +3609,154 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="125" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B1" s="126"/>
       <c r="C1" s="127"/>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="122" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="122" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="122" t="s">
+      <c r="C2" s="122" t="s">
         <v>45</v>
-      </c>
-      <c r="C2" s="122" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="121" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="C3" s="19" t="s">
         <v>48</v>
-      </c>
-      <c r="C3" s="19" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="121" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="18" t="s">
         <v>50</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>51</v>
       </c>
       <c r="C4" s="19"/>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="121" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" s="18" t="s">
         <v>52</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>53</v>
       </c>
       <c r="C5" s="19"/>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="121" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="18" t="s">
         <v>54</v>
-      </c>
-      <c r="B6" s="18" t="s">
-        <v>55</v>
       </c>
       <c r="C6" s="19"/>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="121" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="18" t="s">
         <v>56</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>57</v>
       </c>
       <c r="C7" s="19"/>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="121" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" s="18" t="s">
         <v>58</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>59</v>
       </c>
       <c r="C8" s="19"/>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="121" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9" s="18" t="s">
         <v>60</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>61</v>
       </c>
       <c r="C9" s="19"/>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="121" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="18" t="s">
         <v>62</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>63</v>
       </c>
       <c r="C10" s="19"/>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="121" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" s="18" t="s">
         <v>64</v>
-      </c>
-      <c r="B11" s="18" t="s">
-        <v>65</v>
       </c>
       <c r="C11" s="19"/>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="121" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" s="18" t="s">
         <v>66</v>
-      </c>
-      <c r="B12" s="18" t="s">
-        <v>67</v>
       </c>
       <c r="C12" s="19"/>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="121" t="s">
+        <v>67</v>
+      </c>
+      <c r="B13" s="18" t="s">
         <v>68</v>
-      </c>
-      <c r="B13" s="18" t="s">
-        <v>69</v>
       </c>
       <c r="C13" s="19"/>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="121" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" s="18" t="s">
         <v>70</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>71</v>
       </c>
       <c r="C14" s="19"/>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="121" t="s">
+        <v>71</v>
+      </c>
+      <c r="B15" s="18" t="s">
         <v>72</v>
-      </c>
-      <c r="B15" s="18" t="s">
-        <v>73</v>
       </c>
       <c r="C15" s="19"/>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="121" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="18" t="s">
         <v>74</v>
-      </c>
-      <c r="B16" s="18" t="s">
-        <v>75</v>
       </c>
       <c r="C16" s="19"/>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="19"/>
       <c r="B17" s="18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C17" s="19"/>
     </row>
@@ -3796,7 +3770,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="C20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -3821,7 +3795,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16" customHeight="1">
@@ -3861,16 +3835,16 @@
         <v>5</v>
       </c>
       <c r="B5" s="111" t="s">
+        <v>208</v>
+      </c>
+      <c r="C5" s="112" t="s">
         <v>209</v>
       </c>
-      <c r="C5" s="112" t="s">
+      <c r="D5" s="112" t="s">
         <v>210</v>
       </c>
-      <c r="D5" s="112" t="s">
+      <c r="E5" s="112" t="s">
         <v>211</v>
-      </c>
-      <c r="E5" s="112" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -4558,122 +4532,122 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" t="s">
         <v>78</v>
-      </c>
-      <c r="B1" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B12" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B14" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B15" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -4697,71 +4671,71 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" t="s">
         <v>94</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>95</v>
-      </c>
-      <c r="C1" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" t="s">
         <v>97</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>98</v>
-      </c>
-      <c r="C2" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C3" t="s">
         <v>100</v>
-      </c>
-      <c r="B3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C3" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B4" t="s">
         <v>102</v>
       </c>
-      <c r="B4" t="s">
-        <v>103</v>
-      </c>
       <c r="C4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="46" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -4786,21 +4760,21 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="12" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="77" t="s">
+        <v>109</v>
+      </c>
+      <c r="B3" s="77" t="s">
         <v>110</v>
       </c>
-      <c r="B3" s="77" t="s">
+      <c r="C3" s="77" t="s">
         <v>111</v>
       </c>
-      <c r="C3" s="77" t="s">
+      <c r="D3" s="77" t="s">
         <v>112</v>
-      </c>
-      <c r="D3" s="77" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="80" customHeight="1">
@@ -4808,13 +4782,13 @@
         <v>46196</v>
       </c>
       <c r="B4" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="D4" s="4" t="s">
         <v>115</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -4843,38 +4817,38 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="29" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="16" customHeight="1">
       <c r="A5" s="67" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="67" t="s">
         <v>119</v>
       </c>
-      <c r="B5" s="67" t="s">
+      <c r="C5" s="68" t="s">
         <v>120</v>
       </c>
-      <c r="C5" s="68" t="s">
+      <c r="D5" s="67" t="s">
         <v>121</v>
       </c>
-      <c r="D5" s="67" t="s">
+      <c r="E5" s="67" t="s">
         <v>122</v>
       </c>
-      <c r="E5" s="67" t="s">
+      <c r="F5" s="67" t="s">
         <v>123</v>
       </c>
-      <c r="F5" s="67" t="s">
+      <c r="G5" t="s">
         <v>124</v>
       </c>
-      <c r="G5" t="s">
-        <v>125</v>
-      </c>
       <c r="H5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="16" customHeight="1">
@@ -4883,22 +4857,22 @@
         <v>1</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C6" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="D6" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="F6" s="27" t="s">
         <v>129</v>
       </c>
-      <c r="F6" s="27" t="s">
+      <c r="G6" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>131</v>
       </c>
       <c r="H6" s="1"/>
     </row>
@@ -4908,19 +4882,19 @@
         <v>2</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C7" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C7" s="15" t="s">
-        <v>127</v>
-      </c>
       <c r="D7" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="E7" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="E7" s="15" t="s">
-        <v>133</v>
-      </c>
       <c r="F7" s="27" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
@@ -4931,19 +4905,19 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C8" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C8" s="15" t="s">
-        <v>127</v>
-      </c>
       <c r="D8" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>135</v>
-      </c>
       <c r="F8" s="27" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
@@ -4954,22 +4928,22 @@
         <v>4</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C9" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C9" s="15" t="s">
-        <v>127</v>
-      </c>
       <c r="D9" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F9" s="27" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H9" s="1"/>
     </row>
@@ -4979,22 +4953,22 @@
         <v>5</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C10" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C10" s="15" t="s">
-        <v>127</v>
-      </c>
       <c r="D10" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>138</v>
-      </c>
       <c r="F10" s="27" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H10" s="1"/>
     </row>
@@ -5004,22 +4978,22 @@
         <v>6</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C11" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C11" s="15" t="s">
-        <v>127</v>
-      </c>
       <c r="D11" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E11" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="E11" s="15" t="s">
-        <v>140</v>
-      </c>
       <c r="F11" s="27" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="H11" s="1"/>
     </row>
@@ -5029,16 +5003,16 @@
         <v>7</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C12" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C12" s="15" t="s">
-        <v>127</v>
-      </c>
       <c r="D12" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E12" s="15" t="s">
         <v>141</v>
-      </c>
-      <c r="E12" s="15" t="s">
-        <v>142</v>
       </c>
       <c r="F12" s="27"/>
       <c r="G12" s="1"/>
@@ -5050,16 +5024,16 @@
         <v>8</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C13" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C13" s="15" t="s">
-        <v>127</v>
-      </c>
       <c r="D13" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>144</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="1"/>
@@ -5071,16 +5045,16 @@
         <v>9</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C14" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C14" s="15" t="s">
-        <v>127</v>
-      </c>
       <c r="D14" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>146</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="1"/>
@@ -5092,16 +5066,16 @@
         <v>10</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C15" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C15" s="15" t="s">
-        <v>127</v>
-      </c>
       <c r="D15" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>148</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="1"/>
@@ -5113,16 +5087,16 @@
         <v>11</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C16" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C16" s="15" t="s">
-        <v>127</v>
-      </c>
       <c r="D16" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="E16" s="15" t="s">
         <v>149</v>
-      </c>
-      <c r="E16" s="15" t="s">
-        <v>150</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="1"/>
@@ -5134,16 +5108,16 @@
         <v>12</v>
       </c>
       <c r="B17" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C17" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C17" s="15" t="s">
-        <v>127</v>
-      </c>
       <c r="D17" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="E17" s="15" t="s">
         <v>151</v>
-      </c>
-      <c r="E17" s="15" t="s">
-        <v>152</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="1"/>
@@ -5155,16 +5129,16 @@
         <v>13</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C18" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C18" s="15" t="s">
-        <v>127</v>
-      </c>
       <c r="D18" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E18" s="15" t="s">
         <v>153</v>
-      </c>
-      <c r="E18" s="15" t="s">
-        <v>154</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="1"/>
@@ -5176,16 +5150,16 @@
         <v>14</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C19" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C19" s="15" t="s">
-        <v>127</v>
-      </c>
       <c r="D19" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="E19" s="15" t="s">
         <v>155</v>
-      </c>
-      <c r="E19" s="15" t="s">
-        <v>156</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="1"/>
@@ -5197,16 +5171,16 @@
         <v>15</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C20" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="C20" s="15" t="s">
+      <c r="D20" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="E20" s="15" t="s">
         <v>159</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>160</v>
       </c>
       <c r="F20" s="27"/>
       <c r="G20" s="2"/>
@@ -5218,16 +5192,16 @@
         <v>16</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C21" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="C21" s="15" t="s">
-        <v>158</v>
-      </c>
       <c r="D21" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="E21" s="15" t="s">
         <v>161</v>
-      </c>
-      <c r="E21" s="15" t="s">
-        <v>162</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="2"/>
@@ -5239,16 +5213,16 @@
         <v>17</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C22" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="C22" s="15" t="s">
-        <v>158</v>
-      </c>
       <c r="D22" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="E22" s="15" t="s">
         <v>163</v>
-      </c>
-      <c r="E22" s="15" t="s">
-        <v>164</v>
       </c>
       <c r="F22" s="27"/>
       <c r="G22" s="2"/>
@@ -5260,16 +5234,16 @@
         <v>18</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C23" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="C23" s="15" t="s">
-        <v>158</v>
-      </c>
       <c r="D23" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="E23" s="15" t="s">
         <v>165</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>166</v>
       </c>
       <c r="F23" s="27"/>
       <c r="G23" s="2"/>
@@ -5281,16 +5255,16 @@
         <v>19</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C24" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="C24" s="15" t="s">
+      <c r="D24" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E24" s="15" t="s">
         <v>168</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="E24" s="15" t="s">
-        <v>169</v>
       </c>
       <c r="F24" s="27"/>
       <c r="G24" s="1"/>
@@ -5302,16 +5276,16 @@
         <v>20</v>
       </c>
       <c r="B25" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C25" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="C25" s="15" t="s">
-        <v>168</v>
-      </c>
       <c r="D25" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="1"/>
@@ -5323,16 +5297,16 @@
         <v>21</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C26" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="C26" s="15" t="s">
-        <v>168</v>
-      </c>
       <c r="D26" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="E26" s="15" t="s">
         <v>171</v>
-      </c>
-      <c r="E26" s="15" t="s">
-        <v>172</v>
       </c>
       <c r="F26" s="27"/>
       <c r="G26" s="1"/>
@@ -5344,22 +5318,22 @@
         <v>22</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C27" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="C27" s="15" t="s">
+      <c r="D27" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E27" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="D27" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="E27" s="15" t="s">
-        <v>175</v>
-      </c>
       <c r="F27" s="27" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H27" s="1"/>
     </row>
@@ -5369,19 +5343,19 @@
         <v>23</v>
       </c>
       <c r="B28" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C28" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="C28" s="15" t="s">
-        <v>174</v>
-      </c>
       <c r="D28" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F28" s="27" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
@@ -5428,7 +5402,7 @@
   <sheetData>
     <row r="1" spans="1:19">
       <c r="A1" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B1" s="3"/>
     </row>
@@ -5450,7 +5424,7 @@
     </row>
     <row r="3" spans="1:19">
       <c r="A3" s="78" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B3" s="3"/>
       <c r="P3" s="32" t="str">
@@ -5477,10 +5451,10 @@
     <row r="5" spans="1:19" ht="32" customHeight="1">
       <c r="A5" s="7"/>
       <c r="B5" s="28" t="s">
+        <v>176</v>
+      </c>
+      <c r="C5" s="130" t="s">
         <v>177</v>
-      </c>
-      <c r="C5" s="130" t="s">
-        <v>178</v>
       </c>
       <c r="D5" s="131"/>
       <c r="E5" s="131"/>
@@ -5488,22 +5462,22 @@
       <c r="G5" s="131"/>
       <c r="H5" s="131"/>
       <c r="I5" s="128" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="J5" s="129"/>
       <c r="K5" s="129"/>
       <c r="L5" s="129"/>
       <c r="M5" s="30" t="s">
+        <v>179</v>
+      </c>
+      <c r="N5" s="50" t="s">
         <v>180</v>
       </c>
-      <c r="N5" s="50" t="s">
-        <v>181</v>
-      </c>
       <c r="O5" s="56" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="P5" s="130" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="Q5" s="129"/>
       <c r="R5" s="129"/>
@@ -5511,117 +5485,117 @@
     </row>
     <row r="6" spans="1:19">
       <c r="B6" s="20" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F6" s="26" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G6" s="22" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H6" s="22" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I6" s="24" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="J6" s="24" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K6" s="24" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="L6" s="24" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="M6" s="31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="N6" s="49" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="O6" s="21" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="P6" s="22" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q6" s="22" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="R6" s="22" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="S6" s="22" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="48" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="F7" s="69" t="s">
+        <v>77</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="F7" s="69" t="s">
-        <v>78</v>
-      </c>
-      <c r="G7" s="5" t="s">
+      <c r="H7" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="I7" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="J7" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="K7" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="L7" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="M7" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="M7" s="5" t="s">
+      <c r="N7" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="N7" s="5" t="s">
+      <c r="O7" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="P7" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="O7" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="P7" s="5" t="s">
+      <c r="Q7" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="Q7" s="5" t="s">
+      <c r="R7" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="R7" s="5" t="s">
+      <c r="S7" s="5" t="s">
         <v>196</v>
-      </c>
-      <c r="S7" s="5" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="8" spans="1:19">
@@ -6541,13 +6515,13 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="7" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D1" s="7"/>
     </row>
     <row r="3" spans="1:9" ht="16" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F3" s="70" t="s">
         <v>1</v>
@@ -6564,7 +6538,7 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D4" s="52"/>
       <c r="F4" s="32" t="str">
@@ -6586,31 +6560,31 @@
     </row>
     <row r="6" spans="1:9" ht="16" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>201</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>202</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F6" s="76" t="s">
+        <v>202</v>
+      </c>
+      <c r="G6" s="76" t="s">
         <v>203</v>
       </c>
-      <c r="G6" s="76" t="s">
+      <c r="H6" s="76" t="s">
         <v>204</v>
       </c>
-      <c r="H6" s="76" t="s">
+      <c r="I6" s="76" t="s">
         <v>205</v>
-      </c>
-      <c r="I6" s="76" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -6919,7 +6893,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:AR90"/>
+  <dimension ref="A1:AQ90"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="39.1640625" style="35" bestFit="1" customWidth="1"/>
@@ -6936,61 +6910,60 @@
     <col min="14" max="14" width="8.5" style="37" customWidth="1" outlineLevel="1"/>
     <col min="15" max="16" width="18.33203125" style="37" customWidth="1" outlineLevel="2"/>
     <col min="17" max="17" width="29.5" style="37" customWidth="1" outlineLevel="2"/>
-    <col min="18" max="18" width="24.33203125" style="37" customWidth="1" outlineLevel="2"/>
-    <col min="19" max="19" width="29" style="37" customWidth="1" outlineLevel="2"/>
-    <col min="20" max="21" width="18.33203125" style="37" customWidth="1" outlineLevel="2"/>
-    <col min="22" max="22" width="17.1640625" style="37" customWidth="1" outlineLevel="1"/>
-    <col min="23" max="25" width="9.1640625" style="37" customWidth="1" outlineLevel="2"/>
-    <col min="26" max="26" width="9.1640625" style="35" customWidth="1" outlineLevel="2"/>
-    <col min="27" max="32" width="9.1640625" style="38" customWidth="1" outlineLevel="2"/>
-    <col min="33" max="33" width="19.33203125" style="38" customWidth="1" outlineLevel="1"/>
-    <col min="34" max="37" width="33.33203125" style="38" customWidth="1"/>
-    <col min="38" max="41" width="9" style="38" customWidth="1"/>
-    <col min="42" max="16384" width="9" style="38"/>
+    <col min="18" max="18" width="29" style="37" customWidth="1" outlineLevel="2"/>
+    <col min="19" max="20" width="18.33203125" style="37" customWidth="1" outlineLevel="2"/>
+    <col min="21" max="21" width="17.1640625" style="37" customWidth="1" outlineLevel="1"/>
+    <col min="22" max="24" width="9.1640625" style="37" customWidth="1" outlineLevel="2"/>
+    <col min="25" max="25" width="9.1640625" style="35" customWidth="1" outlineLevel="2"/>
+    <col min="26" max="31" width="9.1640625" style="38" customWidth="1" outlineLevel="2"/>
+    <col min="32" max="32" width="19.33203125" style="38" customWidth="1" outlineLevel="1"/>
+    <col min="33" max="36" width="33.33203125" style="38" customWidth="1"/>
+    <col min="37" max="40" width="9" style="38" customWidth="1"/>
+    <col min="41" max="16384" width="9" style="38"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44">
+    <row r="1" spans="1:43">
       <c r="A1" s="34" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="2" spans="1:44" ht="16" customHeight="1">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="2" spans="1:43" ht="16" customHeight="1">
+      <c r="AG2" s="71" t="s">
+        <v>1</v>
+      </c>
       <c r="AH2" s="71" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI2" s="71" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AJ2" s="71" t="s">
-        <v>3</v>
-      </c>
-      <c r="AK2" s="71" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:44">
+    <row r="3" spans="1:43">
       <c r="A3" s="52"/>
-      <c r="AH3" s="32" t="str">
+      <c r="AG3" s="32" t="str">
         <f>IF('General Settings'!$G$11=0,"",'General Settings'!$G$11)</f>
         <v>en</v>
       </c>
+      <c r="AH3" s="32" t="str">
+        <f>IF('General Settings'!$G$12=0,"",'General Settings'!$G$12)</f>
+        <v/>
+      </c>
       <c r="AI3" s="32" t="str">
-        <f>IF('General Settings'!$G$12=0,"",'General Settings'!$G$12)</f>
+        <f>IF('General Settings'!$G$13=0,"",'General Settings'!$G$13)</f>
         <v/>
       </c>
       <c r="AJ3" s="32" t="str">
-        <f>IF('General Settings'!$G$13=0,"",'General Settings'!$G$13)</f>
-        <v/>
-      </c>
-      <c r="AK3" s="32" t="str">
         <f>IF('General Settings'!$G$14=0,"",'General Settings'!$G$14)</f>
         <v/>
       </c>
     </row>
-    <row r="4" spans="1:44">
+    <row r="4" spans="1:43">
       <c r="A4" s="34"/>
     </row>
-    <row r="5" spans="1:44" s="40" customFormat="1" ht="45" customHeight="1">
+    <row r="5" spans="1:43" s="40" customFormat="1" ht="45" customHeight="1">
       <c r="A5" s="39" t="s">
         <v>5</v>
       </c>
@@ -7087,10 +7060,10 @@
       <c r="AF5" s="74" t="s">
         <v>36</v>
       </c>
-      <c r="AG5" s="74" t="s">
+      <c r="AG5" s="73" t="s">
         <v>37</v>
       </c>
-      <c r="AH5" s="73" t="s">
+      <c r="AH5" s="75" t="s">
         <v>38</v>
       </c>
       <c r="AI5" s="75" t="s">
@@ -7099,12 +7072,9 @@
       <c r="AJ5" s="75" t="s">
         <v>40</v>
       </c>
-      <c r="AK5" s="75" t="s">
-        <v>41</v>
-      </c>
-      <c r="AR5" s="41"/>
-    </row>
-    <row r="6" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AQ5" s="41"/>
+    </row>
+    <row r="6" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A6" s="6"/>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -7139,15 +7109,14 @@
       <c r="AC6" s="8"/>
       <c r="AD6" s="8"/>
       <c r="AE6" s="8"/>
-      <c r="AF6" s="8"/>
-      <c r="AG6" s="25"/>
-      <c r="AH6" s="42"/>
-      <c r="AI6" s="54"/>
-      <c r="AJ6" s="42"/>
-      <c r="AK6" s="39"/>
-      <c r="AR6" s="41"/>
-    </row>
-    <row r="7" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AF6" s="25"/>
+      <c r="AG6" s="42"/>
+      <c r="AH6" s="54"/>
+      <c r="AI6" s="42"/>
+      <c r="AJ6" s="39"/>
+      <c r="AQ6" s="41"/>
+    </row>
+    <row r="7" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -7182,15 +7151,14 @@
       <c r="AC7" s="8"/>
       <c r="AD7" s="8"/>
       <c r="AE7" s="8"/>
-      <c r="AF7" s="8"/>
-      <c r="AG7" s="25"/>
+      <c r="AF7" s="25"/>
+      <c r="AG7" s="6"/>
       <c r="AH7" s="6"/>
-      <c r="AI7" s="6"/>
-      <c r="AJ7" s="42"/>
-      <c r="AK7" s="39"/>
-      <c r="AR7" s="41"/>
-    </row>
-    <row r="8" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AI7" s="42"/>
+      <c r="AJ7" s="39"/>
+      <c r="AQ7" s="41"/>
+    </row>
+    <row r="8" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -7225,15 +7193,14 @@
       <c r="AC8" s="8"/>
       <c r="AD8" s="8"/>
       <c r="AE8" s="8"/>
-      <c r="AF8" s="8"/>
-      <c r="AG8" s="25"/>
+      <c r="AF8" s="25"/>
+      <c r="AG8" s="6"/>
       <c r="AH8" s="6"/>
-      <c r="AI8" s="6"/>
-      <c r="AJ8" s="42"/>
-      <c r="AK8" s="39"/>
-      <c r="AR8" s="41"/>
-    </row>
-    <row r="9" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AI8" s="42"/>
+      <c r="AJ8" s="39"/>
+      <c r="AQ8" s="41"/>
+    </row>
+    <row r="9" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -7268,15 +7235,14 @@
       <c r="AC9" s="8"/>
       <c r="AD9" s="8"/>
       <c r="AE9" s="8"/>
-      <c r="AF9" s="8"/>
-      <c r="AG9" s="25"/>
+      <c r="AF9" s="25"/>
+      <c r="AG9" s="6"/>
       <c r="AH9" s="6"/>
-      <c r="AI9" s="6"/>
-      <c r="AJ9" s="42"/>
-      <c r="AK9" s="39"/>
-      <c r="AR9" s="41"/>
-    </row>
-    <row r="10" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AI9" s="42"/>
+      <c r="AJ9" s="39"/>
+      <c r="AQ9" s="41"/>
+    </row>
+    <row r="10" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A10" s="42"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -7300,8 +7266,8 @@
       <c r="R10" s="8"/>
       <c r="S10" s="8"/>
       <c r="T10" s="8"/>
-      <c r="U10" s="8"/>
-      <c r="V10" s="9"/>
+      <c r="U10" s="9"/>
+      <c r="V10" s="8"/>
       <c r="W10" s="8"/>
       <c r="X10" s="8"/>
       <c r="Y10" s="8"/>
@@ -7311,15 +7277,14 @@
       <c r="AC10" s="8"/>
       <c r="AD10" s="8"/>
       <c r="AE10" s="8"/>
-      <c r="AF10" s="8"/>
-      <c r="AG10" s="25"/>
+      <c r="AF10" s="25"/>
+      <c r="AG10" s="6"/>
       <c r="AH10" s="6"/>
-      <c r="AI10" s="6"/>
-      <c r="AJ10" s="42"/>
-      <c r="AK10" s="39"/>
-      <c r="AR10" s="41"/>
-    </row>
-    <row r="11" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AI10" s="42"/>
+      <c r="AJ10" s="39"/>
+      <c r="AQ10" s="41"/>
+    </row>
+    <row r="11" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A11" s="42"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -7343,8 +7308,8 @@
       <c r="R11" s="8"/>
       <c r="S11" s="8"/>
       <c r="T11" s="8"/>
-      <c r="U11" s="8"/>
-      <c r="V11" s="9"/>
+      <c r="U11" s="9"/>
+      <c r="V11" s="8"/>
       <c r="W11" s="8"/>
       <c r="X11" s="8"/>
       <c r="Y11" s="8"/>
@@ -7354,15 +7319,14 @@
       <c r="AC11" s="8"/>
       <c r="AD11" s="8"/>
       <c r="AE11" s="8"/>
-      <c r="AF11" s="8"/>
-      <c r="AG11" s="25"/>
+      <c r="AF11" s="25"/>
+      <c r="AG11" s="6"/>
       <c r="AH11" s="6"/>
-      <c r="AI11" s="6"/>
-      <c r="AJ11" s="42"/>
-      <c r="AK11" s="39"/>
-      <c r="AR11" s="41"/>
-    </row>
-    <row r="12" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AI11" s="42"/>
+      <c r="AJ11" s="39"/>
+      <c r="AQ11" s="41"/>
+    </row>
+    <row r="12" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A12" s="6"/>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -7397,15 +7361,14 @@
       <c r="AC12" s="8"/>
       <c r="AD12" s="8"/>
       <c r="AE12" s="8"/>
-      <c r="AF12" s="8"/>
-      <c r="AG12" s="25"/>
-      <c r="AH12" s="42"/>
-      <c r="AI12" s="54"/>
-      <c r="AJ12" s="42"/>
-      <c r="AK12" s="39"/>
-      <c r="AR12" s="41"/>
-    </row>
-    <row r="13" spans="1:44">
+      <c r="AF12" s="25"/>
+      <c r="AG12" s="42"/>
+      <c r="AH12" s="54"/>
+      <c r="AI12" s="42"/>
+      <c r="AJ12" s="39"/>
+      <c r="AQ12" s="41"/>
+    </row>
+    <row r="13" spans="1:43">
       <c r="A13" s="6"/>
       <c r="B13" s="42"/>
       <c r="C13" s="42"/>
@@ -7440,14 +7403,13 @@
       <c r="AC13" s="8"/>
       <c r="AD13" s="8"/>
       <c r="AE13" s="8"/>
-      <c r="AF13" s="8"/>
-      <c r="AG13" s="25"/>
-      <c r="AH13" s="6"/>
+      <c r="AF13" s="25"/>
+      <c r="AG13" s="6"/>
+      <c r="AH13" s="42"/>
       <c r="AI13" s="42"/>
-      <c r="AJ13" s="42"/>
-      <c r="AK13" s="39"/>
-    </row>
-    <row r="14" spans="1:44">
+      <c r="AJ13" s="39"/>
+    </row>
+    <row r="14" spans="1:43">
       <c r="A14" s="42"/>
       <c r="B14" s="42"/>
       <c r="C14" s="6"/>
@@ -7482,14 +7444,13 @@
       <c r="AC14" s="8"/>
       <c r="AD14" s="8"/>
       <c r="AE14" s="8"/>
-      <c r="AF14" s="8"/>
-      <c r="AG14" s="25"/>
+      <c r="AF14" s="25"/>
+      <c r="AG14" s="42"/>
       <c r="AH14" s="42"/>
       <c r="AI14" s="42"/>
-      <c r="AJ14" s="42"/>
-      <c r="AK14" s="39"/>
-    </row>
-    <row r="15" spans="1:44">
+      <c r="AJ14" s="39"/>
+    </row>
+    <row r="15" spans="1:43">
       <c r="A15" s="42"/>
       <c r="B15" s="42"/>
       <c r="C15" s="6"/>
@@ -7524,14 +7485,13 @@
       <c r="AC15" s="8"/>
       <c r="AD15" s="8"/>
       <c r="AE15" s="8"/>
-      <c r="AF15" s="8"/>
-      <c r="AG15" s="25"/>
+      <c r="AF15" s="25"/>
+      <c r="AG15" s="42"/>
       <c r="AH15" s="42"/>
       <c r="AI15" s="42"/>
-      <c r="AJ15" s="42"/>
-      <c r="AK15" s="39"/>
-    </row>
-    <row r="16" spans="1:44">
+      <c r="AJ15" s="39"/>
+    </row>
+    <row r="16" spans="1:43">
       <c r="A16" s="42"/>
       <c r="B16" s="42"/>
       <c r="C16" s="6"/>
@@ -7566,14 +7526,13 @@
       <c r="AC16" s="8"/>
       <c r="AD16" s="8"/>
       <c r="AE16" s="8"/>
-      <c r="AF16" s="8"/>
-      <c r="AG16" s="25"/>
-      <c r="AH16" s="42"/>
-      <c r="AI16" s="6"/>
-      <c r="AJ16" s="42"/>
-      <c r="AK16" s="39"/>
-    </row>
-    <row r="17" spans="1:44">
+      <c r="AF16" s="25"/>
+      <c r="AG16" s="42"/>
+      <c r="AH16" s="6"/>
+      <c r="AI16" s="42"/>
+      <c r="AJ16" s="39"/>
+    </row>
+    <row r="17" spans="1:43">
       <c r="A17" s="42"/>
       <c r="B17" s="42"/>
       <c r="C17" s="6"/>
@@ -7608,14 +7567,13 @@
       <c r="AC17" s="8"/>
       <c r="AD17" s="8"/>
       <c r="AE17" s="8"/>
-      <c r="AF17" s="8"/>
-      <c r="AG17" s="25"/>
-      <c r="AH17" s="42"/>
-      <c r="AI17" s="6"/>
-      <c r="AJ17" s="42"/>
-      <c r="AK17" s="39"/>
-    </row>
-    <row r="18" spans="1:44">
+      <c r="AF17" s="25"/>
+      <c r="AG17" s="42"/>
+      <c r="AH17" s="6"/>
+      <c r="AI17" s="42"/>
+      <c r="AJ17" s="39"/>
+    </row>
+    <row r="18" spans="1:43">
       <c r="A18" s="42"/>
       <c r="B18" s="42"/>
       <c r="C18" s="42"/>
@@ -7650,14 +7608,13 @@
       <c r="AC18" s="8"/>
       <c r="AD18" s="8"/>
       <c r="AE18" s="8"/>
-      <c r="AF18" s="8"/>
-      <c r="AG18" s="25"/>
-      <c r="AH18" s="42"/>
-      <c r="AI18" s="6"/>
-      <c r="AJ18" s="42"/>
-      <c r="AK18" s="39"/>
-    </row>
-    <row r="19" spans="1:44">
+      <c r="AF18" s="25"/>
+      <c r="AG18" s="42"/>
+      <c r="AH18" s="6"/>
+      <c r="AI18" s="42"/>
+      <c r="AJ18" s="39"/>
+    </row>
+    <row r="19" spans="1:43">
       <c r="A19" s="42"/>
       <c r="B19" s="6"/>
       <c r="C19" s="42"/>
@@ -7692,14 +7649,13 @@
       <c r="AC19" s="8"/>
       <c r="AD19" s="8"/>
       <c r="AE19" s="8"/>
-      <c r="AF19" s="8"/>
-      <c r="AG19" s="25"/>
+      <c r="AF19" s="25"/>
+      <c r="AG19" s="6"/>
       <c r="AH19" s="6"/>
-      <c r="AI19" s="6"/>
-      <c r="AJ19" s="42"/>
-      <c r="AK19" s="39"/>
-    </row>
-    <row r="20" spans="1:44">
+      <c r="AI19" s="42"/>
+      <c r="AJ19" s="39"/>
+    </row>
+    <row r="20" spans="1:43">
       <c r="A20" s="42"/>
       <c r="B20" s="6"/>
       <c r="C20" s="42"/>
@@ -7734,14 +7690,13 @@
       <c r="AC20" s="8"/>
       <c r="AD20" s="8"/>
       <c r="AE20" s="8"/>
-      <c r="AF20" s="8"/>
-      <c r="AG20" s="25"/>
-      <c r="AH20" s="42"/>
-      <c r="AI20" s="6"/>
-      <c r="AJ20" s="42"/>
-      <c r="AK20" s="39"/>
-    </row>
-    <row r="21" spans="1:44">
+      <c r="AF20" s="25"/>
+      <c r="AG20" s="42"/>
+      <c r="AH20" s="6"/>
+      <c r="AI20" s="42"/>
+      <c r="AJ20" s="39"/>
+    </row>
+    <row r="21" spans="1:43">
       <c r="A21" s="42"/>
       <c r="B21" s="6"/>
       <c r="C21" s="42"/>
@@ -7776,14 +7731,13 @@
       <c r="AC21" s="8"/>
       <c r="AD21" s="8"/>
       <c r="AE21" s="8"/>
-      <c r="AF21" s="8"/>
-      <c r="AG21" s="25"/>
-      <c r="AH21" s="42"/>
-      <c r="AI21" s="6"/>
-      <c r="AJ21" s="42"/>
-      <c r="AK21" s="39"/>
-    </row>
-    <row r="22" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AF21" s="25"/>
+      <c r="AG21" s="42"/>
+      <c r="AH21" s="6"/>
+      <c r="AI21" s="42"/>
+      <c r="AJ21" s="39"/>
+    </row>
+    <row r="22" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A22" s="42"/>
       <c r="B22" s="42"/>
       <c r="C22" s="6"/>
@@ -7807,8 +7761,8 @@
       <c r="R22" s="8"/>
       <c r="S22" s="8"/>
       <c r="T22" s="8"/>
-      <c r="U22" s="8"/>
-      <c r="V22" s="9"/>
+      <c r="U22" s="9"/>
+      <c r="V22" s="8"/>
       <c r="W22" s="8"/>
       <c r="X22" s="8"/>
       <c r="Y22" s="8"/>
@@ -7818,15 +7772,14 @@
       <c r="AC22" s="8"/>
       <c r="AD22" s="8"/>
       <c r="AE22" s="8"/>
-      <c r="AF22" s="8"/>
-      <c r="AG22" s="25"/>
-      <c r="AH22" s="42"/>
-      <c r="AI22" s="51"/>
-      <c r="AJ22" s="42"/>
-      <c r="AK22" s="39"/>
-      <c r="AR22" s="41"/>
-    </row>
-    <row r="23" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AF22" s="25"/>
+      <c r="AG22" s="42"/>
+      <c r="AH22" s="51"/>
+      <c r="AI22" s="42"/>
+      <c r="AJ22" s="39"/>
+      <c r="AQ22" s="41"/>
+    </row>
+    <row r="23" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A23" s="42"/>
       <c r="B23" s="42"/>
       <c r="C23" s="6"/>
@@ -7853,7 +7806,7 @@
       <c r="U23" s="8"/>
       <c r="V23" s="8"/>
       <c r="W23" s="8"/>
-      <c r="X23" s="8"/>
+      <c r="X23" s="44"/>
       <c r="Y23" s="44"/>
       <c r="Z23" s="44"/>
       <c r="AA23" s="44"/>
@@ -7861,15 +7814,14 @@
       <c r="AC23" s="44"/>
       <c r="AD23" s="44"/>
       <c r="AE23" s="44"/>
-      <c r="AF23" s="44"/>
-      <c r="AG23" s="60"/>
-      <c r="AH23" s="42"/>
-      <c r="AI23" s="51"/>
-      <c r="AJ23" s="42"/>
-      <c r="AK23" s="39"/>
-      <c r="AR23" s="41"/>
-    </row>
-    <row r="24" spans="1:44">
+      <c r="AF23" s="60"/>
+      <c r="AG23" s="42"/>
+      <c r="AH23" s="51"/>
+      <c r="AI23" s="42"/>
+      <c r="AJ23" s="39"/>
+      <c r="AQ23" s="41"/>
+    </row>
+    <row r="24" spans="1:43">
       <c r="A24" s="42"/>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -7890,10 +7842,10 @@
       <c r="O24" s="8"/>
       <c r="P24" s="8"/>
       <c r="Q24" s="8"/>
-      <c r="R24" s="8"/>
+      <c r="R24" s="53"/>
       <c r="S24" s="53"/>
       <c r="T24" s="53"/>
-      <c r="U24" s="53"/>
+      <c r="U24" s="8"/>
       <c r="V24" s="8"/>
       <c r="W24" s="8"/>
       <c r="X24" s="8"/>
@@ -7904,12 +7856,11 @@
       <c r="AC24" s="8"/>
       <c r="AD24" s="8"/>
       <c r="AE24" s="8"/>
-      <c r="AF24" s="8"/>
-      <c r="AG24" s="25"/>
-      <c r="AH24" s="6"/>
-      <c r="AI24" s="63"/>
-    </row>
-    <row r="25" spans="1:44">
+      <c r="AF24" s="25"/>
+      <c r="AG24" s="6"/>
+      <c r="AH24" s="63"/>
+    </row>
+    <row r="25" spans="1:43">
       <c r="A25" s="42"/>
       <c r="B25" s="42"/>
       <c r="C25" s="6"/>
@@ -7944,14 +7895,13 @@
       <c r="AC25" s="8"/>
       <c r="AD25" s="8"/>
       <c r="AE25" s="8"/>
-      <c r="AF25" s="8"/>
-      <c r="AG25" s="25"/>
-      <c r="AH25" s="42"/>
-      <c r="AI25" s="6"/>
-      <c r="AJ25" s="42"/>
-      <c r="AK25" s="39"/>
-    </row>
-    <row r="26" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AF25" s="25"/>
+      <c r="AG25" s="42"/>
+      <c r="AH25" s="6"/>
+      <c r="AI25" s="42"/>
+      <c r="AJ25" s="39"/>
+    </row>
+    <row r="26" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A26" s="42"/>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
@@ -7978,7 +7928,7 @@
       <c r="U26" s="8"/>
       <c r="V26" s="8"/>
       <c r="W26" s="8"/>
-      <c r="X26" s="8"/>
+      <c r="X26" s="44"/>
       <c r="Y26" s="44"/>
       <c r="Z26" s="44"/>
       <c r="AA26" s="44"/>
@@ -7986,15 +7936,14 @@
       <c r="AC26" s="44"/>
       <c r="AD26" s="44"/>
       <c r="AE26" s="44"/>
-      <c r="AF26" s="44"/>
-      <c r="AG26" s="60"/>
-      <c r="AH26" s="42"/>
-      <c r="AI26" s="6"/>
-      <c r="AJ26" s="42"/>
-      <c r="AK26" s="39"/>
-      <c r="AR26" s="41"/>
-    </row>
-    <row r="27" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AF26" s="60"/>
+      <c r="AG26" s="42"/>
+      <c r="AH26" s="6"/>
+      <c r="AI26" s="42"/>
+      <c r="AJ26" s="39"/>
+      <c r="AQ26" s="41"/>
+    </row>
+    <row r="27" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A27" s="42"/>
       <c r="B27" s="51"/>
       <c r="C27" s="6"/>
@@ -8021,7 +7970,7 @@
       <c r="U27" s="8"/>
       <c r="V27" s="8"/>
       <c r="W27" s="8"/>
-      <c r="X27" s="8"/>
+      <c r="X27" s="44"/>
       <c r="Y27" s="44"/>
       <c r="Z27" s="44"/>
       <c r="AA27" s="44"/>
@@ -8029,15 +7978,14 @@
       <c r="AC27" s="44"/>
       <c r="AD27" s="44"/>
       <c r="AE27" s="44"/>
-      <c r="AF27" s="44"/>
-      <c r="AG27" s="60"/>
-      <c r="AH27" s="51"/>
-      <c r="AI27" s="6"/>
-      <c r="AJ27" s="42"/>
-      <c r="AK27" s="39"/>
-      <c r="AR27" s="41"/>
-    </row>
-    <row r="28" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AF27" s="60"/>
+      <c r="AG27" s="51"/>
+      <c r="AH27" s="6"/>
+      <c r="AI27" s="42"/>
+      <c r="AJ27" s="39"/>
+      <c r="AQ27" s="41"/>
+    </row>
+    <row r="28" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A28" s="6"/>
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
@@ -8064,7 +8012,7 @@
       <c r="U28" s="8"/>
       <c r="V28" s="8"/>
       <c r="W28" s="8"/>
-      <c r="X28" s="8"/>
+      <c r="X28" s="44"/>
       <c r="Y28" s="44"/>
       <c r="Z28" s="44"/>
       <c r="AA28" s="44"/>
@@ -8072,15 +8020,14 @@
       <c r="AC28" s="44"/>
       <c r="AD28" s="44"/>
       <c r="AE28" s="44"/>
-      <c r="AF28" s="44"/>
-      <c r="AG28" s="60"/>
+      <c r="AF28" s="60"/>
+      <c r="AG28" s="42"/>
       <c r="AH28" s="42"/>
       <c r="AI28" s="42"/>
-      <c r="AJ28" s="42"/>
-      <c r="AK28" s="39"/>
-      <c r="AR28" s="41"/>
-    </row>
-    <row r="29" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AJ28" s="39"/>
+      <c r="AQ28" s="41"/>
+    </row>
+    <row r="29" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A29" s="6"/>
       <c r="B29" s="6"/>
       <c r="C29" s="6"/>
@@ -8101,13 +8048,13 @@
       <c r="O29" s="8"/>
       <c r="P29" s="8"/>
       <c r="Q29" s="8"/>
-      <c r="R29" s="8"/>
+      <c r="R29" s="53"/>
       <c r="S29" s="53"/>
-      <c r="T29" s="53"/>
+      <c r="T29" s="8"/>
       <c r="U29" s="8"/>
       <c r="V29" s="8"/>
       <c r="W29" s="8"/>
-      <c r="X29" s="8"/>
+      <c r="X29" s="44"/>
       <c r="Y29" s="44"/>
       <c r="Z29" s="44"/>
       <c r="AA29" s="44"/>
@@ -8115,15 +8062,14 @@
       <c r="AC29" s="44"/>
       <c r="AD29" s="44"/>
       <c r="AE29" s="44"/>
-      <c r="AF29" s="44"/>
-      <c r="AG29" s="60"/>
-      <c r="AH29" s="6"/>
-      <c r="AI29" s="63"/>
-      <c r="AJ29" s="42"/>
-      <c r="AK29" s="39"/>
-      <c r="AR29" s="41"/>
-    </row>
-    <row r="30" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AF29" s="60"/>
+      <c r="AG29" s="6"/>
+      <c r="AH29" s="63"/>
+      <c r="AI29" s="42"/>
+      <c r="AJ29" s="39"/>
+      <c r="AQ29" s="41"/>
+    </row>
+    <row r="30" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A30" s="6"/>
       <c r="B30" s="51"/>
       <c r="C30" s="6"/>
@@ -8150,7 +8096,7 @@
       <c r="U30" s="8"/>
       <c r="V30" s="8"/>
       <c r="W30" s="8"/>
-      <c r="X30" s="8"/>
+      <c r="X30" s="44"/>
       <c r="Y30" s="44"/>
       <c r="Z30" s="44"/>
       <c r="AA30" s="44"/>
@@ -8158,15 +8104,14 @@
       <c r="AC30" s="44"/>
       <c r="AD30" s="44"/>
       <c r="AE30" s="44"/>
-      <c r="AF30" s="44"/>
-      <c r="AG30" s="60"/>
+      <c r="AF30" s="60"/>
+      <c r="AG30" s="51"/>
       <c r="AH30" s="51"/>
-      <c r="AI30" s="51"/>
-      <c r="AJ30" s="42"/>
-      <c r="AK30" s="39"/>
-      <c r="AR30" s="41"/>
-    </row>
-    <row r="31" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AI30" s="42"/>
+      <c r="AJ30" s="39"/>
+      <c r="AQ30" s="41"/>
+    </row>
+    <row r="31" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A31" s="6"/>
       <c r="B31" s="51"/>
       <c r="C31" s="6"/>
@@ -8193,7 +8138,7 @@
       <c r="U31" s="8"/>
       <c r="V31" s="8"/>
       <c r="W31" s="8"/>
-      <c r="X31" s="8"/>
+      <c r="X31" s="44"/>
       <c r="Y31" s="44"/>
       <c r="Z31" s="44"/>
       <c r="AA31" s="44"/>
@@ -8201,15 +8146,14 @@
       <c r="AC31" s="44"/>
       <c r="AD31" s="44"/>
       <c r="AE31" s="44"/>
-      <c r="AF31" s="44"/>
-      <c r="AG31" s="60"/>
+      <c r="AF31" s="60"/>
+      <c r="AG31" s="51"/>
       <c r="AH31" s="51"/>
-      <c r="AI31" s="51"/>
-      <c r="AJ31" s="42"/>
-      <c r="AK31" s="39"/>
-      <c r="AR31" s="41"/>
-    </row>
-    <row r="32" spans="1:44">
+      <c r="AI31" s="42"/>
+      <c r="AJ31" s="39"/>
+      <c r="AQ31" s="41"/>
+    </row>
+    <row r="32" spans="1:43">
       <c r="A32" s="42"/>
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
@@ -8244,14 +8188,13 @@
       <c r="AC32" s="8"/>
       <c r="AD32" s="8"/>
       <c r="AE32" s="8"/>
-      <c r="AF32" s="8"/>
-      <c r="AG32" s="25"/>
-      <c r="AH32" s="42"/>
-      <c r="AI32" s="54"/>
-      <c r="AJ32" s="42"/>
-      <c r="AK32" s="39"/>
-    </row>
-    <row r="33" spans="1:44">
+      <c r="AF32" s="25"/>
+      <c r="AG32" s="42"/>
+      <c r="AH32" s="54"/>
+      <c r="AI32" s="42"/>
+      <c r="AJ32" s="39"/>
+    </row>
+    <row r="33" spans="1:43">
       <c r="A33" s="42"/>
       <c r="B33" s="6"/>
       <c r="C33" s="6"/>
@@ -8272,10 +8215,10 @@
       <c r="O33" s="8"/>
       <c r="P33" s="8"/>
       <c r="Q33" s="8"/>
-      <c r="R33" s="8"/>
+      <c r="R33" s="53"/>
       <c r="S33" s="53"/>
       <c r="T33" s="53"/>
-      <c r="U33" s="53"/>
+      <c r="U33" s="8"/>
       <c r="V33" s="8"/>
       <c r="W33" s="8"/>
       <c r="X33" s="8"/>
@@ -8286,14 +8229,13 @@
       <c r="AC33" s="8"/>
       <c r="AD33" s="8"/>
       <c r="AE33" s="8"/>
-      <c r="AF33" s="8"/>
-      <c r="AG33" s="25"/>
-      <c r="AH33" s="6"/>
-      <c r="AI33" s="63"/>
-      <c r="AJ33" s="42"/>
-      <c r="AK33" s="39"/>
-    </row>
-    <row r="34" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AF33" s="25"/>
+      <c r="AG33" s="6"/>
+      <c r="AH33" s="63"/>
+      <c r="AI33" s="42"/>
+      <c r="AJ33" s="39"/>
+    </row>
+    <row r="34" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A34" s="42"/>
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
@@ -8328,15 +8270,14 @@
       <c r="AC34" s="8"/>
       <c r="AD34" s="8"/>
       <c r="AE34" s="8"/>
-      <c r="AF34" s="8"/>
-      <c r="AG34" s="25"/>
+      <c r="AF34" s="25"/>
+      <c r="AG34" s="6"/>
       <c r="AH34" s="6"/>
-      <c r="AI34" s="6"/>
-      <c r="AJ34" s="42"/>
-      <c r="AK34" s="39"/>
-      <c r="AR34" s="41"/>
-    </row>
-    <row r="35" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AI34" s="42"/>
+      <c r="AJ34" s="39"/>
+      <c r="AQ34" s="41"/>
+    </row>
+    <row r="35" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A35" s="42"/>
       <c r="B35" s="6"/>
       <c r="C35" s="6"/>
@@ -8371,15 +8312,14 @@
       <c r="AC35" s="8"/>
       <c r="AD35" s="8"/>
       <c r="AE35" s="8"/>
-      <c r="AF35" s="8"/>
-      <c r="AG35" s="25"/>
+      <c r="AF35" s="25"/>
+      <c r="AG35" s="6"/>
       <c r="AH35" s="6"/>
-      <c r="AI35" s="6"/>
-      <c r="AJ35" s="42"/>
-      <c r="AK35" s="39"/>
-      <c r="AR35" s="41"/>
-    </row>
-    <row r="36" spans="1:44" s="40" customFormat="1" ht="14" customHeight="1">
+      <c r="AI35" s="42"/>
+      <c r="AJ35" s="39"/>
+      <c r="AQ35" s="41"/>
+    </row>
+    <row r="36" spans="1:43" s="40" customFormat="1" ht="14" customHeight="1">
       <c r="A36" s="42"/>
       <c r="B36" s="6"/>
       <c r="C36" s="6"/>
@@ -8414,15 +8354,14 @@
       <c r="AC36" s="8"/>
       <c r="AD36" s="8"/>
       <c r="AE36" s="8"/>
-      <c r="AF36" s="8"/>
-      <c r="AG36" s="25"/>
+      <c r="AF36" s="25"/>
+      <c r="AG36" s="6"/>
       <c r="AH36" s="6"/>
-      <c r="AI36" s="6"/>
-      <c r="AJ36" s="42"/>
-      <c r="AK36" s="39"/>
-      <c r="AR36" s="41"/>
-    </row>
-    <row r="37" spans="1:44" ht="160" customHeight="1">
+      <c r="AI36" s="42"/>
+      <c r="AJ36" s="39"/>
+      <c r="AQ36" s="41"/>
+    </row>
+    <row r="37" spans="1:43" ht="160" customHeight="1">
       <c r="A37" s="42"/>
       <c r="B37" s="6"/>
       <c r="C37" s="42"/>
@@ -8457,14 +8396,13 @@
       <c r="AC37" s="8"/>
       <c r="AD37" s="8"/>
       <c r="AE37" s="8"/>
-      <c r="AF37" s="8"/>
-      <c r="AG37" s="25"/>
+      <c r="AF37" s="25"/>
+      <c r="AG37" s="42"/>
       <c r="AH37" s="42"/>
       <c r="AI37" s="42"/>
-      <c r="AJ37" s="42"/>
-      <c r="AK37" s="39"/>
-    </row>
-    <row r="38" spans="1:44">
+      <c r="AJ37" s="39"/>
+    </row>
+    <row r="38" spans="1:43">
       <c r="A38" s="42"/>
       <c r="B38" s="6"/>
       <c r="C38" s="42"/>
@@ -8499,14 +8437,13 @@
       <c r="AC38" s="8"/>
       <c r="AD38" s="8"/>
       <c r="AE38" s="8"/>
-      <c r="AF38" s="8"/>
-      <c r="AG38" s="25"/>
+      <c r="AF38" s="25"/>
+      <c r="AG38" s="42"/>
       <c r="AH38" s="42"/>
       <c r="AI38" s="42"/>
-      <c r="AJ38" s="42"/>
-      <c r="AK38" s="39"/>
-    </row>
-    <row r="39" spans="1:44">
+      <c r="AJ38" s="39"/>
+    </row>
+    <row r="39" spans="1:43">
       <c r="A39" s="42"/>
       <c r="B39" s="6"/>
       <c r="C39" s="42"/>
@@ -8541,14 +8478,13 @@
       <c r="AC39" s="8"/>
       <c r="AD39" s="8"/>
       <c r="AE39" s="8"/>
-      <c r="AF39" s="8"/>
-      <c r="AG39" s="25"/>
-      <c r="AH39" s="42"/>
-      <c r="AI39" s="63"/>
-      <c r="AJ39" s="42"/>
-      <c r="AK39" s="39"/>
-    </row>
-    <row r="40" spans="1:44">
+      <c r="AF39" s="25"/>
+      <c r="AG39" s="42"/>
+      <c r="AH39" s="63"/>
+      <c r="AI39" s="42"/>
+      <c r="AJ39" s="39"/>
+    </row>
+    <row r="40" spans="1:43">
       <c r="A40" s="42"/>
       <c r="B40" s="6"/>
       <c r="C40" s="42"/>
@@ -8583,14 +8519,13 @@
       <c r="AC40" s="8"/>
       <c r="AD40" s="8"/>
       <c r="AE40" s="8"/>
-      <c r="AF40" s="8"/>
-      <c r="AG40" s="25"/>
-      <c r="AH40" s="42"/>
-      <c r="AI40" s="63"/>
-      <c r="AJ40" s="42"/>
-      <c r="AK40" s="39"/>
-    </row>
-    <row r="41" spans="1:44">
+      <c r="AF40" s="25"/>
+      <c r="AG40" s="42"/>
+      <c r="AH40" s="63"/>
+      <c r="AI40" s="42"/>
+      <c r="AJ40" s="39"/>
+    </row>
+    <row r="41" spans="1:43">
       <c r="A41" s="42"/>
       <c r="B41" s="6"/>
       <c r="C41" s="42"/>
@@ -8625,14 +8560,13 @@
       <c r="AC41" s="8"/>
       <c r="AD41" s="8"/>
       <c r="AE41" s="8"/>
-      <c r="AF41" s="8"/>
-      <c r="AG41" s="25"/>
-      <c r="AH41" s="42"/>
-      <c r="AI41" s="63"/>
-      <c r="AJ41" s="42"/>
-      <c r="AK41" s="39"/>
-    </row>
-    <row r="42" spans="1:44">
+      <c r="AF41" s="25"/>
+      <c r="AG41" s="42"/>
+      <c r="AH41" s="63"/>
+      <c r="AI41" s="42"/>
+      <c r="AJ41" s="39"/>
+    </row>
+    <row r="42" spans="1:43">
       <c r="A42" s="42"/>
       <c r="B42" s="6"/>
       <c r="C42" s="42"/>
@@ -8667,14 +8601,13 @@
       <c r="AC42" s="8"/>
       <c r="AD42" s="8"/>
       <c r="AE42" s="8"/>
-      <c r="AF42" s="8"/>
-      <c r="AG42" s="25"/>
-      <c r="AH42" s="42"/>
-      <c r="AI42" s="63"/>
-      <c r="AJ42" s="42"/>
-      <c r="AK42" s="39"/>
-    </row>
-    <row r="43" spans="1:44">
+      <c r="AF42" s="25"/>
+      <c r="AG42" s="42"/>
+      <c r="AH42" s="63"/>
+      <c r="AI42" s="42"/>
+      <c r="AJ42" s="39"/>
+    </row>
+    <row r="43" spans="1:43">
       <c r="A43" s="42"/>
       <c r="B43" s="6"/>
       <c r="C43" s="6"/>
@@ -8709,14 +8642,13 @@
       <c r="AC43" s="8"/>
       <c r="AD43" s="8"/>
       <c r="AE43" s="8"/>
-      <c r="AF43" s="8"/>
-      <c r="AG43" s="25"/>
-      <c r="AH43" s="42"/>
-      <c r="AI43" s="54"/>
-      <c r="AJ43" s="42"/>
-      <c r="AK43" s="39"/>
-    </row>
-    <row r="44" spans="1:44">
+      <c r="AF43" s="25"/>
+      <c r="AG43" s="42"/>
+      <c r="AH43" s="54"/>
+      <c r="AI43" s="42"/>
+      <c r="AJ43" s="39"/>
+    </row>
+    <row r="44" spans="1:43">
       <c r="A44" s="42"/>
       <c r="B44" s="6"/>
       <c r="C44" s="6"/>
@@ -8737,10 +8669,10 @@
       <c r="O44" s="8"/>
       <c r="P44" s="8"/>
       <c r="Q44" s="8"/>
-      <c r="R44" s="8"/>
-      <c r="S44" s="42"/>
+      <c r="R44" s="42"/>
+      <c r="S44" s="53"/>
       <c r="T44" s="53"/>
-      <c r="U44" s="53"/>
+      <c r="U44" s="8"/>
       <c r="V44" s="8"/>
       <c r="W44" s="8"/>
       <c r="X44" s="8"/>
@@ -8751,14 +8683,13 @@
       <c r="AC44" s="8"/>
       <c r="AD44" s="8"/>
       <c r="AE44" s="8"/>
-      <c r="AF44" s="8"/>
-      <c r="AG44" s="25"/>
-      <c r="AH44" s="6"/>
-      <c r="AI44" s="63"/>
-      <c r="AJ44" s="42"/>
-      <c r="AK44" s="39"/>
-    </row>
-    <row r="45" spans="1:44">
+      <c r="AF44" s="25"/>
+      <c r="AG44" s="6"/>
+      <c r="AH44" s="63"/>
+      <c r="AI44" s="42"/>
+      <c r="AJ44" s="39"/>
+    </row>
+    <row r="45" spans="1:43">
       <c r="A45" s="42"/>
       <c r="B45" s="6"/>
       <c r="C45" s="6"/>
@@ -8779,10 +8710,10 @@
       <c r="O45" s="8"/>
       <c r="P45" s="8"/>
       <c r="Q45" s="8"/>
-      <c r="R45" s="8"/>
+      <c r="R45" s="53"/>
       <c r="S45" s="53"/>
       <c r="T45" s="53"/>
-      <c r="U45" s="53"/>
+      <c r="U45" s="8"/>
       <c r="V45" s="8"/>
       <c r="W45" s="8"/>
       <c r="X45" s="8"/>
@@ -8793,14 +8724,13 @@
       <c r="AC45" s="8"/>
       <c r="AD45" s="8"/>
       <c r="AE45" s="8"/>
-      <c r="AF45" s="8"/>
-      <c r="AG45" s="25"/>
-      <c r="AH45" s="42"/>
-      <c r="AI45" s="63"/>
-      <c r="AJ45" s="42"/>
-      <c r="AK45" s="39"/>
-    </row>
-    <row r="46" spans="1:44">
+      <c r="AF45" s="25"/>
+      <c r="AG45" s="42"/>
+      <c r="AH45" s="63"/>
+      <c r="AI45" s="42"/>
+      <c r="AJ45" s="39"/>
+    </row>
+    <row r="46" spans="1:43">
       <c r="A46" s="42"/>
       <c r="B46" s="6"/>
       <c r="C46" s="6"/>
@@ -8835,14 +8765,13 @@
       <c r="AC46" s="8"/>
       <c r="AD46" s="8"/>
       <c r="AE46" s="8"/>
-      <c r="AF46" s="8"/>
-      <c r="AG46" s="25"/>
-      <c r="AH46" s="42"/>
-      <c r="AI46" s="63"/>
-      <c r="AJ46" s="42"/>
-      <c r="AK46" s="39"/>
-    </row>
-    <row r="47" spans="1:44">
+      <c r="AF46" s="25"/>
+      <c r="AG46" s="42"/>
+      <c r="AH46" s="63"/>
+      <c r="AI46" s="42"/>
+      <c r="AJ46" s="39"/>
+    </row>
+    <row r="47" spans="1:43">
       <c r="A47" s="42"/>
       <c r="B47" s="61"/>
       <c r="C47" s="42"/>
@@ -8877,14 +8806,13 @@
       <c r="AC47" s="8"/>
       <c r="AD47" s="8"/>
       <c r="AE47" s="8"/>
-      <c r="AF47" s="8"/>
-      <c r="AG47" s="25"/>
+      <c r="AF47" s="25"/>
+      <c r="AG47" s="61"/>
       <c r="AH47" s="61"/>
-      <c r="AI47" s="61"/>
-      <c r="AJ47" s="42"/>
-      <c r="AK47" s="39"/>
-    </row>
-    <row r="48" spans="1:44">
+      <c r="AI47" s="42"/>
+      <c r="AJ47" s="39"/>
+    </row>
+    <row r="48" spans="1:43">
       <c r="A48" s="42"/>
       <c r="B48" s="6"/>
       <c r="C48" s="6"/>
@@ -8919,14 +8847,13 @@
       <c r="AC48" s="8"/>
       <c r="AD48" s="8"/>
       <c r="AE48" s="8"/>
-      <c r="AF48" s="8"/>
-      <c r="AG48" s="25"/>
-      <c r="AH48" s="42"/>
-      <c r="AI48" s="54"/>
-      <c r="AJ48" s="42"/>
-      <c r="AK48" s="39"/>
-    </row>
-    <row r="49" spans="1:37">
+      <c r="AF48" s="25"/>
+      <c r="AG48" s="42"/>
+      <c r="AH48" s="54"/>
+      <c r="AI48" s="42"/>
+      <c r="AJ48" s="39"/>
+    </row>
+    <row r="49" spans="1:36">
       <c r="A49" s="42"/>
       <c r="B49" s="6"/>
       <c r="C49" s="6"/>
@@ -8947,10 +8874,10 @@
       <c r="O49" s="8"/>
       <c r="P49" s="8"/>
       <c r="Q49" s="8"/>
-      <c r="R49" s="8"/>
+      <c r="R49" s="53"/>
       <c r="S49" s="53"/>
       <c r="T49" s="53"/>
-      <c r="U49" s="53"/>
+      <c r="U49" s="8"/>
       <c r="V49" s="8"/>
       <c r="W49" s="8"/>
       <c r="X49" s="8"/>
@@ -8961,14 +8888,13 @@
       <c r="AC49" s="8"/>
       <c r="AD49" s="8"/>
       <c r="AE49" s="8"/>
-      <c r="AF49" s="8"/>
-      <c r="AG49" s="25"/>
-      <c r="AH49" s="6"/>
-      <c r="AI49" s="63"/>
-      <c r="AJ49" s="42"/>
-      <c r="AK49" s="39"/>
-    </row>
-    <row r="50" spans="1:37">
+      <c r="AF49" s="25"/>
+      <c r="AG49" s="6"/>
+      <c r="AH49" s="63"/>
+      <c r="AI49" s="42"/>
+      <c r="AJ49" s="39"/>
+    </row>
+    <row r="50" spans="1:36">
       <c r="A50" s="42"/>
       <c r="B50" s="6"/>
       <c r="C50" s="6"/>
@@ -8989,9 +8915,9 @@
       <c r="O50" s="8"/>
       <c r="P50" s="8"/>
       <c r="Q50" s="8"/>
-      <c r="R50" s="8"/>
+      <c r="R50" s="53"/>
       <c r="S50" s="53"/>
-      <c r="T50" s="53"/>
+      <c r="T50" s="8"/>
       <c r="U50" s="8"/>
       <c r="V50" s="8"/>
       <c r="W50" s="8"/>
@@ -9003,14 +8929,13 @@
       <c r="AC50" s="8"/>
       <c r="AD50" s="8"/>
       <c r="AE50" s="8"/>
-      <c r="AF50" s="8"/>
-      <c r="AG50" s="25"/>
-      <c r="AH50" s="42"/>
-      <c r="AI50" s="63"/>
-      <c r="AJ50" s="42"/>
-      <c r="AK50" s="39"/>
-    </row>
-    <row r="51" spans="1:37">
+      <c r="AF50" s="25"/>
+      <c r="AG50" s="42"/>
+      <c r="AH50" s="63"/>
+      <c r="AI50" s="42"/>
+      <c r="AJ50" s="39"/>
+    </row>
+    <row r="51" spans="1:36">
       <c r="A51" s="42"/>
       <c r="B51" s="6"/>
       <c r="C51" s="6"/>
@@ -9045,14 +8970,13 @@
       <c r="AC51" s="8"/>
       <c r="AD51" s="8"/>
       <c r="AE51" s="8"/>
-      <c r="AF51" s="8"/>
-      <c r="AG51" s="25"/>
-      <c r="AH51" s="6"/>
-      <c r="AI51" s="63"/>
-      <c r="AJ51" s="42"/>
-      <c r="AK51" s="39"/>
-    </row>
-    <row r="52" spans="1:37">
+      <c r="AF51" s="25"/>
+      <c r="AG51" s="6"/>
+      <c r="AH51" s="63"/>
+      <c r="AI51" s="42"/>
+      <c r="AJ51" s="39"/>
+    </row>
+    <row r="52" spans="1:36">
       <c r="A52" s="42"/>
       <c r="B52" s="6"/>
       <c r="C52" s="6"/>
@@ -9087,14 +9011,13 @@
       <c r="AC52" s="8"/>
       <c r="AD52" s="8"/>
       <c r="AE52" s="8"/>
-      <c r="AF52" s="8"/>
-      <c r="AG52" s="25"/>
-      <c r="AH52" s="6"/>
-      <c r="AI52" s="63"/>
-      <c r="AJ52" s="42"/>
-      <c r="AK52" s="39"/>
-    </row>
-    <row r="53" spans="1:37">
+      <c r="AF52" s="25"/>
+      <c r="AG52" s="6"/>
+      <c r="AH52" s="63"/>
+      <c r="AI52" s="42"/>
+      <c r="AJ52" s="39"/>
+    </row>
+    <row r="53" spans="1:36">
       <c r="A53" s="42"/>
       <c r="B53" s="6"/>
       <c r="C53" s="6"/>
@@ -9129,14 +9052,13 @@
       <c r="AC53" s="8"/>
       <c r="AD53" s="8"/>
       <c r="AE53" s="8"/>
-      <c r="AF53" s="8"/>
-      <c r="AG53" s="25"/>
-      <c r="AH53" s="42"/>
-      <c r="AI53" s="54"/>
-      <c r="AJ53" s="42"/>
-      <c r="AK53" s="39"/>
-    </row>
-    <row r="54" spans="1:37">
+      <c r="AF53" s="25"/>
+      <c r="AG53" s="42"/>
+      <c r="AH53" s="54"/>
+      <c r="AI53" s="42"/>
+      <c r="AJ53" s="39"/>
+    </row>
+    <row r="54" spans="1:36">
       <c r="A54" s="42"/>
       <c r="B54" s="6"/>
       <c r="C54" s="6"/>
@@ -9157,10 +9079,10 @@
       <c r="O54" s="8"/>
       <c r="P54" s="8"/>
       <c r="Q54" s="8"/>
-      <c r="R54" s="8"/>
+      <c r="R54" s="53"/>
       <c r="S54" s="53"/>
       <c r="T54" s="53"/>
-      <c r="U54" s="53"/>
+      <c r="U54" s="8"/>
       <c r="V54" s="8"/>
       <c r="W54" s="8"/>
       <c r="X54" s="8"/>
@@ -9171,14 +9093,13 @@
       <c r="AC54" s="8"/>
       <c r="AD54" s="8"/>
       <c r="AE54" s="8"/>
-      <c r="AF54" s="8"/>
-      <c r="AG54" s="25"/>
-      <c r="AH54" s="6"/>
-      <c r="AI54" s="63"/>
-      <c r="AJ54" s="42"/>
-      <c r="AK54" s="39"/>
-    </row>
-    <row r="55" spans="1:37">
+      <c r="AF54" s="25"/>
+      <c r="AG54" s="6"/>
+      <c r="AH54" s="63"/>
+      <c r="AI54" s="42"/>
+      <c r="AJ54" s="39"/>
+    </row>
+    <row r="55" spans="1:36">
       <c r="A55" s="42"/>
       <c r="B55" s="6"/>
       <c r="C55" s="42"/>
@@ -9213,14 +9134,13 @@
       <c r="AC55" s="8"/>
       <c r="AD55" s="8"/>
       <c r="AE55" s="8"/>
-      <c r="AF55" s="8"/>
-      <c r="AG55" s="25"/>
+      <c r="AF55" s="25"/>
+      <c r="AG55" s="42"/>
       <c r="AH55" s="42"/>
       <c r="AI55" s="42"/>
-      <c r="AJ55" s="42"/>
-      <c r="AK55" s="39"/>
-    </row>
-    <row r="56" spans="1:37">
+      <c r="AJ55" s="39"/>
+    </row>
+    <row r="56" spans="1:36">
       <c r="A56" s="42"/>
       <c r="B56" s="42"/>
       <c r="C56" s="42"/>
@@ -9241,10 +9161,10 @@
       <c r="O56" s="8"/>
       <c r="P56" s="8"/>
       <c r="Q56" s="8"/>
-      <c r="R56" s="8"/>
+      <c r="R56" s="53"/>
       <c r="S56" s="53"/>
       <c r="T56" s="53"/>
-      <c r="U56" s="53"/>
+      <c r="U56" s="8"/>
       <c r="V56" s="8"/>
       <c r="W56" s="8"/>
       <c r="X56" s="8"/>
@@ -9255,14 +9175,13 @@
       <c r="AC56" s="8"/>
       <c r="AD56" s="8"/>
       <c r="AE56" s="8"/>
-      <c r="AF56" s="8"/>
-      <c r="AG56" s="25"/>
+      <c r="AF56" s="25"/>
+      <c r="AG56" s="42"/>
       <c r="AH56" s="42"/>
       <c r="AI56" s="42"/>
-      <c r="AJ56" s="42"/>
-      <c r="AK56" s="39"/>
-    </row>
-    <row r="57" spans="1:37">
+      <c r="AJ56" s="39"/>
+    </row>
+    <row r="57" spans="1:36">
       <c r="A57" s="42"/>
       <c r="B57" s="6"/>
       <c r="C57" s="42"/>
@@ -9297,14 +9216,13 @@
       <c r="AC57" s="8"/>
       <c r="AD57" s="8"/>
       <c r="AE57" s="8"/>
-      <c r="AF57" s="8"/>
-      <c r="AG57" s="25"/>
+      <c r="AF57" s="25"/>
+      <c r="AG57" s="42"/>
       <c r="AH57" s="42"/>
       <c r="AI57" s="42"/>
-      <c r="AJ57" s="42"/>
-      <c r="AK57" s="39"/>
-    </row>
-    <row r="58" spans="1:37">
+      <c r="AJ57" s="39"/>
+    </row>
+    <row r="58" spans="1:36">
       <c r="A58" s="42"/>
       <c r="B58" s="6"/>
       <c r="C58" s="42"/>
@@ -9339,14 +9257,13 @@
       <c r="AC58" s="8"/>
       <c r="AD58" s="8"/>
       <c r="AE58" s="8"/>
-      <c r="AF58" s="8"/>
-      <c r="AG58" s="25"/>
-      <c r="AH58" s="42"/>
-      <c r="AI58" s="63"/>
-      <c r="AJ58" s="42"/>
-      <c r="AK58" s="39"/>
-    </row>
-    <row r="59" spans="1:37">
+      <c r="AF58" s="25"/>
+      <c r="AG58" s="42"/>
+      <c r="AH58" s="63"/>
+      <c r="AI58" s="42"/>
+      <c r="AJ58" s="39"/>
+    </row>
+    <row r="59" spans="1:36">
       <c r="A59" s="42"/>
       <c r="B59" s="6"/>
       <c r="C59" s="42"/>
@@ -9381,14 +9298,13 @@
       <c r="AC59" s="8"/>
       <c r="AD59" s="8"/>
       <c r="AE59" s="8"/>
-      <c r="AF59" s="8"/>
-      <c r="AG59" s="25"/>
-      <c r="AH59" s="42"/>
-      <c r="AI59" s="63"/>
-      <c r="AJ59" s="42"/>
-      <c r="AK59" s="39"/>
-    </row>
-    <row r="60" spans="1:37">
+      <c r="AF59" s="25"/>
+      <c r="AG59" s="42"/>
+      <c r="AH59" s="63"/>
+      <c r="AI59" s="42"/>
+      <c r="AJ59" s="39"/>
+    </row>
+    <row r="60" spans="1:36">
       <c r="A60" s="42"/>
       <c r="B60" s="6"/>
       <c r="C60" s="6"/>
@@ -9423,14 +9339,13 @@
       <c r="AC60" s="8"/>
       <c r="AD60" s="8"/>
       <c r="AE60" s="8"/>
-      <c r="AF60" s="8"/>
-      <c r="AG60" s="25"/>
-      <c r="AH60" s="42"/>
-      <c r="AI60" s="54"/>
-      <c r="AJ60" s="42"/>
-      <c r="AK60" s="39"/>
-    </row>
-    <row r="61" spans="1:37">
+      <c r="AF60" s="25"/>
+      <c r="AG60" s="42"/>
+      <c r="AH60" s="54"/>
+      <c r="AI60" s="42"/>
+      <c r="AJ60" s="39"/>
+    </row>
+    <row r="61" spans="1:36">
       <c r="A61" s="42"/>
       <c r="B61" s="6"/>
       <c r="C61" s="6"/>
@@ -9451,10 +9366,10 @@
       <c r="O61" s="8"/>
       <c r="P61" s="8"/>
       <c r="Q61" s="8"/>
-      <c r="R61" s="8"/>
+      <c r="R61" s="53"/>
       <c r="S61" s="53"/>
       <c r="T61" s="53"/>
-      <c r="U61" s="53"/>
+      <c r="U61" s="8"/>
       <c r="V61" s="8"/>
       <c r="W61" s="8"/>
       <c r="X61" s="8"/>
@@ -9465,14 +9380,13 @@
       <c r="AC61" s="8"/>
       <c r="AD61" s="8"/>
       <c r="AE61" s="8"/>
-      <c r="AF61" s="8"/>
-      <c r="AG61" s="25"/>
-      <c r="AH61" s="6"/>
-      <c r="AI61" s="63"/>
-      <c r="AJ61" s="42"/>
-      <c r="AK61" s="39"/>
-    </row>
-    <row r="62" spans="1:37">
+      <c r="AF61" s="25"/>
+      <c r="AG61" s="6"/>
+      <c r="AH61" s="63"/>
+      <c r="AI61" s="42"/>
+      <c r="AJ61" s="39"/>
+    </row>
+    <row r="62" spans="1:36">
       <c r="A62" s="42"/>
       <c r="B62" s="42"/>
       <c r="C62" s="42"/>
@@ -9493,10 +9407,10 @@
       <c r="O62" s="8"/>
       <c r="P62" s="8"/>
       <c r="Q62" s="8"/>
-      <c r="R62" s="8"/>
+      <c r="R62" s="53"/>
       <c r="S62" s="53"/>
       <c r="T62" s="53"/>
-      <c r="U62" s="53"/>
+      <c r="U62" s="8"/>
       <c r="V62" s="8"/>
       <c r="W62" s="8"/>
       <c r="X62" s="8"/>
@@ -9507,14 +9421,13 @@
       <c r="AC62" s="8"/>
       <c r="AD62" s="8"/>
       <c r="AE62" s="8"/>
-      <c r="AF62" s="8"/>
-      <c r="AG62" s="25"/>
+      <c r="AF62" s="25"/>
+      <c r="AG62" s="42"/>
       <c r="AH62" s="42"/>
       <c r="AI62" s="42"/>
-      <c r="AJ62" s="42"/>
-      <c r="AK62" s="39"/>
-    </row>
-    <row r="63" spans="1:37">
+      <c r="AJ62" s="39"/>
+    </row>
+    <row r="63" spans="1:36">
       <c r="A63" s="42"/>
       <c r="B63" s="42"/>
       <c r="C63" s="42"/>
@@ -9535,9 +9448,9 @@
       <c r="O63" s="8"/>
       <c r="P63" s="8"/>
       <c r="Q63" s="8"/>
-      <c r="R63" s="8"/>
+      <c r="R63" s="53"/>
       <c r="S63" s="53"/>
-      <c r="T63" s="53"/>
+      <c r="T63" s="8"/>
       <c r="U63" s="8"/>
       <c r="V63" s="8"/>
       <c r="W63" s="8"/>
@@ -9549,14 +9462,13 @@
       <c r="AC63" s="8"/>
       <c r="AD63" s="8"/>
       <c r="AE63" s="8"/>
-      <c r="AF63" s="8"/>
-      <c r="AG63" s="25"/>
+      <c r="AF63" s="25"/>
+      <c r="AG63" s="42"/>
       <c r="AH63" s="42"/>
       <c r="AI63" s="42"/>
-      <c r="AJ63" s="42"/>
-      <c r="AK63" s="39"/>
-    </row>
-    <row r="64" spans="1:37">
+      <c r="AJ63" s="39"/>
+    </row>
+    <row r="64" spans="1:36">
       <c r="A64" s="42"/>
       <c r="B64" s="42"/>
       <c r="C64" s="42"/>
@@ -9591,14 +9503,13 @@
       <c r="AC64" s="8"/>
       <c r="AD64" s="8"/>
       <c r="AE64" s="8"/>
-      <c r="AF64" s="8"/>
-      <c r="AG64" s="25"/>
+      <c r="AF64" s="25"/>
+      <c r="AG64" s="42"/>
       <c r="AH64" s="42"/>
       <c r="AI64" s="42"/>
-      <c r="AJ64" s="42"/>
-      <c r="AK64" s="39"/>
-    </row>
-    <row r="65" spans="1:37" ht="16" customHeight="1">
+      <c r="AJ64" s="39"/>
+    </row>
+    <row r="65" spans="1:36" ht="16" customHeight="1">
       <c r="A65" s="42"/>
       <c r="B65" s="42"/>
       <c r="C65" s="42"/>
@@ -9625,7 +9536,7 @@
       <c r="U65" s="8"/>
       <c r="V65" s="8"/>
       <c r="W65" s="8"/>
-      <c r="X65" s="8"/>
+      <c r="X65" s="39"/>
       <c r="Y65" s="39"/>
       <c r="Z65" s="39"/>
       <c r="AA65" s="39"/>
@@ -9633,14 +9544,13 @@
       <c r="AC65" s="39"/>
       <c r="AD65" s="39"/>
       <c r="AE65" s="39"/>
-      <c r="AF65" s="39"/>
-      <c r="AG65" s="48"/>
-      <c r="AH65" s="42"/>
-      <c r="AI65" s="6"/>
-      <c r="AJ65" s="42"/>
-      <c r="AK65" s="39"/>
-    </row>
-    <row r="66" spans="1:37">
+      <c r="AF65" s="48"/>
+      <c r="AG65" s="42"/>
+      <c r="AH65" s="6"/>
+      <c r="AI65" s="42"/>
+      <c r="AJ65" s="39"/>
+    </row>
+    <row r="66" spans="1:36">
       <c r="A66" s="42"/>
       <c r="B66" s="42"/>
       <c r="C66" s="42"/>
@@ -9667,7 +9577,7 @@
       <c r="U66" s="8"/>
       <c r="V66" s="8"/>
       <c r="W66" s="8"/>
-      <c r="X66" s="8"/>
+      <c r="X66" s="39"/>
       <c r="Y66" s="39"/>
       <c r="Z66" s="39"/>
       <c r="AA66" s="39"/>
@@ -9675,14 +9585,13 @@
       <c r="AC66" s="39"/>
       <c r="AD66" s="39"/>
       <c r="AE66" s="39"/>
-      <c r="AF66" s="39"/>
-      <c r="AG66" s="48"/>
-      <c r="AH66" s="42"/>
-      <c r="AI66" s="6"/>
-      <c r="AJ66" s="42"/>
-      <c r="AK66" s="39"/>
-    </row>
-    <row r="67" spans="1:37">
+      <c r="AF66" s="48"/>
+      <c r="AG66" s="42"/>
+      <c r="AH66" s="6"/>
+      <c r="AI66" s="42"/>
+      <c r="AJ66" s="39"/>
+    </row>
+    <row r="67" spans="1:36">
       <c r="A67" s="42"/>
       <c r="B67" s="42"/>
       <c r="C67" s="42"/>
@@ -9709,7 +9618,7 @@
       <c r="U67" s="8"/>
       <c r="V67" s="8"/>
       <c r="W67" s="8"/>
-      <c r="X67" s="8"/>
+      <c r="X67" s="39"/>
       <c r="Y67" s="39"/>
       <c r="Z67" s="39"/>
       <c r="AA67" s="39"/>
@@ -9717,14 +9626,13 @@
       <c r="AC67" s="39"/>
       <c r="AD67" s="39"/>
       <c r="AE67" s="39"/>
-      <c r="AF67" s="39"/>
-      <c r="AG67" s="48"/>
-      <c r="AH67" s="42"/>
-      <c r="AI67" s="6"/>
-      <c r="AJ67" s="42"/>
-      <c r="AK67" s="39"/>
-    </row>
-    <row r="68" spans="1:37" ht="48" customHeight="1">
+      <c r="AF67" s="48"/>
+      <c r="AG67" s="42"/>
+      <c r="AH67" s="6"/>
+      <c r="AI67" s="42"/>
+      <c r="AJ67" s="39"/>
+    </row>
+    <row r="68" spans="1:36" ht="48" customHeight="1">
       <c r="A68" s="42"/>
       <c r="B68" s="61"/>
       <c r="C68" s="61"/>
@@ -9745,10 +9653,10 @@
       <c r="O68" s="8"/>
       <c r="P68" s="8"/>
       <c r="Q68" s="8"/>
-      <c r="R68" s="8"/>
+      <c r="R68" s="53"/>
       <c r="S68" s="53"/>
       <c r="T68" s="53"/>
-      <c r="U68" s="53"/>
+      <c r="U68" s="8"/>
       <c r="V68" s="8"/>
       <c r="W68" s="8"/>
       <c r="X68" s="8"/>
@@ -9759,14 +9667,13 @@
       <c r="AC68" s="8"/>
       <c r="AD68" s="8"/>
       <c r="AE68" s="8"/>
-      <c r="AF68" s="8"/>
-      <c r="AG68" s="25"/>
-      <c r="AH68" s="61"/>
+      <c r="AF68" s="25"/>
+      <c r="AG68" s="61"/>
+      <c r="AH68" s="42"/>
       <c r="AI68" s="42"/>
-      <c r="AJ68" s="42"/>
-      <c r="AK68" s="39"/>
-    </row>
-    <row r="69" spans="1:37" ht="240" customHeight="1">
+      <c r="AJ68" s="39"/>
+    </row>
+    <row r="69" spans="1:36" ht="240" customHeight="1">
       <c r="A69" s="42"/>
       <c r="B69" s="42"/>
       <c r="C69" s="42"/>
@@ -9801,14 +9708,13 @@
       <c r="AC69" s="8"/>
       <c r="AD69" s="8"/>
       <c r="AE69" s="8"/>
-      <c r="AF69" s="8"/>
-      <c r="AG69" s="48"/>
+      <c r="AF69" s="48"/>
+      <c r="AG69" s="42"/>
       <c r="AH69" s="42"/>
       <c r="AI69" s="42"/>
-      <c r="AJ69" s="42"/>
-      <c r="AK69" s="39"/>
-    </row>
-    <row r="70" spans="1:37">
+      <c r="AJ69" s="39"/>
+    </row>
+    <row r="70" spans="1:36">
       <c r="A70" s="42"/>
       <c r="B70" s="42"/>
       <c r="C70" s="42"/>
@@ -9829,10 +9735,10 @@
       <c r="O70" s="8"/>
       <c r="P70" s="8"/>
       <c r="Q70" s="8"/>
-      <c r="R70" s="8"/>
+      <c r="R70" s="53"/>
       <c r="S70" s="53"/>
       <c r="T70" s="53"/>
-      <c r="U70" s="53"/>
+      <c r="U70" s="8"/>
       <c r="V70" s="8"/>
       <c r="W70" s="8"/>
       <c r="X70" s="8"/>
@@ -9843,14 +9749,13 @@
       <c r="AC70" s="8"/>
       <c r="AD70" s="8"/>
       <c r="AE70" s="8"/>
-      <c r="AF70" s="8"/>
-      <c r="AG70" s="25"/>
+      <c r="AF70" s="25"/>
+      <c r="AG70" s="42"/>
       <c r="AH70" s="42"/>
       <c r="AI70" s="42"/>
-      <c r="AJ70" s="42"/>
-      <c r="AK70" s="39"/>
-    </row>
-    <row r="71" spans="1:37">
+      <c r="AJ70" s="39"/>
+    </row>
+    <row r="71" spans="1:36">
       <c r="A71" s="42"/>
       <c r="B71" s="42"/>
       <c r="C71" s="42"/>
@@ -9885,14 +9790,13 @@
       <c r="AC71" s="8"/>
       <c r="AD71" s="8"/>
       <c r="AE71" s="8"/>
-      <c r="AF71" s="8"/>
-      <c r="AG71" s="25"/>
+      <c r="AF71" s="25"/>
+      <c r="AG71" s="42"/>
       <c r="AH71" s="42"/>
       <c r="AI71" s="42"/>
-      <c r="AJ71" s="42"/>
-      <c r="AK71" s="39"/>
-    </row>
-    <row r="72" spans="1:37">
+      <c r="AJ71" s="39"/>
+    </row>
+    <row r="72" spans="1:36">
       <c r="A72" s="42"/>
       <c r="B72" s="42"/>
       <c r="C72" s="42"/>
@@ -9913,10 +9817,10 @@
       <c r="O72" s="8"/>
       <c r="P72" s="8"/>
       <c r="Q72" s="8"/>
-      <c r="R72" s="8"/>
-      <c r="S72" s="42"/>
+      <c r="R72" s="42"/>
+      <c r="S72" s="53"/>
       <c r="T72" s="53"/>
-      <c r="U72" s="53"/>
+      <c r="U72" s="8"/>
       <c r="V72" s="8"/>
       <c r="W72" s="8"/>
       <c r="X72" s="8"/>
@@ -9927,14 +9831,13 @@
       <c r="AC72" s="8"/>
       <c r="AD72" s="8"/>
       <c r="AE72" s="8"/>
-      <c r="AF72" s="8"/>
-      <c r="AG72" s="25"/>
+      <c r="AF72" s="25"/>
+      <c r="AG72" s="42"/>
       <c r="AH72" s="42"/>
       <c r="AI72" s="42"/>
-      <c r="AJ72" s="42"/>
-      <c r="AK72" s="39"/>
-    </row>
-    <row r="73" spans="1:37" ht="48" customHeight="1">
+      <c r="AJ72" s="39"/>
+    </row>
+    <row r="73" spans="1:36" ht="48" customHeight="1">
       <c r="A73" s="42"/>
       <c r="B73" s="42"/>
       <c r="C73" s="42"/>
@@ -9955,10 +9858,10 @@
       <c r="O73" s="8"/>
       <c r="P73" s="8"/>
       <c r="Q73" s="8"/>
-      <c r="R73" s="8"/>
-      <c r="S73" s="42"/>
+      <c r="R73" s="42"/>
+      <c r="S73" s="53"/>
       <c r="T73" s="53"/>
-      <c r="U73" s="53"/>
+      <c r="U73" s="8"/>
       <c r="V73" s="8"/>
       <c r="W73" s="8"/>
       <c r="X73" s="8"/>
@@ -9969,14 +9872,13 @@
       <c r="AC73" s="8"/>
       <c r="AD73" s="8"/>
       <c r="AE73" s="8"/>
-      <c r="AF73" s="8"/>
-      <c r="AG73" s="25"/>
+      <c r="AF73" s="25"/>
+      <c r="AG73" s="42"/>
       <c r="AH73" s="42"/>
       <c r="AI73" s="42"/>
-      <c r="AJ73" s="42"/>
-      <c r="AK73" s="39"/>
-    </row>
-    <row r="74" spans="1:37">
+      <c r="AJ73" s="39"/>
+    </row>
+    <row r="74" spans="1:36">
       <c r="A74" s="61"/>
       <c r="B74" s="62"/>
       <c r="C74" s="62"/>
@@ -10011,14 +9913,13 @@
       <c r="AC74" s="65"/>
       <c r="AD74" s="65"/>
       <c r="AE74" s="65"/>
-      <c r="AF74" s="65"/>
-      <c r="AG74" s="59"/>
-      <c r="AH74" s="42"/>
-      <c r="AI74" s="66"/>
-      <c r="AJ74" s="42"/>
-      <c r="AK74" s="39"/>
-    </row>
-    <row r="75" spans="1:37">
+      <c r="AF74" s="59"/>
+      <c r="AG74" s="42"/>
+      <c r="AH74" s="66"/>
+      <c r="AI74" s="42"/>
+      <c r="AJ74" s="39"/>
+    </row>
+    <row r="75" spans="1:36">
       <c r="A75" s="61"/>
       <c r="B75" s="6"/>
       <c r="C75" s="6"/>
@@ -10039,10 +9940,10 @@
       <c r="O75" s="8"/>
       <c r="P75" s="8"/>
       <c r="Q75" s="8"/>
-      <c r="R75" s="8"/>
+      <c r="R75" s="53"/>
       <c r="S75" s="53"/>
       <c r="T75" s="53"/>
-      <c r="U75" s="53"/>
+      <c r="U75" s="8"/>
       <c r="V75" s="8"/>
       <c r="W75" s="8"/>
       <c r="X75" s="8"/>
@@ -10053,14 +9954,13 @@
       <c r="AC75" s="8"/>
       <c r="AD75" s="8"/>
       <c r="AE75" s="8"/>
-      <c r="AF75" s="8"/>
-      <c r="AG75" s="25"/>
-      <c r="AH75" s="6"/>
-      <c r="AI75" s="63"/>
-      <c r="AJ75" s="42"/>
-      <c r="AK75" s="39"/>
-    </row>
-    <row r="76" spans="1:37">
+      <c r="AF75" s="25"/>
+      <c r="AG75" s="6"/>
+      <c r="AH75" s="63"/>
+      <c r="AI75" s="42"/>
+      <c r="AJ75" s="39"/>
+    </row>
+    <row r="76" spans="1:36">
       <c r="A76" s="61"/>
       <c r="B76" s="61"/>
       <c r="C76" s="61"/>
@@ -10081,10 +9981,10 @@
       <c r="O76" s="8"/>
       <c r="P76" s="8"/>
       <c r="Q76" s="8"/>
-      <c r="R76" s="8"/>
+      <c r="R76" s="53"/>
       <c r="S76" s="53"/>
       <c r="T76" s="53"/>
-      <c r="U76" s="53"/>
+      <c r="U76" s="65"/>
       <c r="V76" s="65"/>
       <c r="W76" s="65"/>
       <c r="X76" s="65"/>
@@ -10095,14 +9995,13 @@
       <c r="AC76" s="65"/>
       <c r="AD76" s="65"/>
       <c r="AE76" s="65"/>
-      <c r="AF76" s="65"/>
-      <c r="AG76" s="59"/>
-      <c r="AH76" s="61"/>
-      <c r="AI76" s="66"/>
-      <c r="AJ76" s="42"/>
-      <c r="AK76" s="39"/>
-    </row>
-    <row r="77" spans="1:37" ht="48" customHeight="1">
+      <c r="AF76" s="59"/>
+      <c r="AG76" s="61"/>
+      <c r="AH76" s="66"/>
+      <c r="AI76" s="42"/>
+      <c r="AJ76" s="39"/>
+    </row>
+    <row r="77" spans="1:36" ht="48" customHeight="1">
       <c r="A77" s="61"/>
       <c r="B77" s="61"/>
       <c r="C77" s="61"/>
@@ -10123,10 +10022,10 @@
       <c r="O77" s="8"/>
       <c r="P77" s="8"/>
       <c r="Q77" s="8"/>
-      <c r="R77" s="8"/>
+      <c r="R77" s="53"/>
       <c r="S77" s="53"/>
       <c r="T77" s="53"/>
-      <c r="U77" s="53"/>
+      <c r="U77" s="8"/>
       <c r="V77" s="8"/>
       <c r="W77" s="8"/>
       <c r="X77" s="8"/>
@@ -10137,14 +10036,13 @@
       <c r="AC77" s="8"/>
       <c r="AD77" s="8"/>
       <c r="AE77" s="8"/>
-      <c r="AF77" s="8"/>
-      <c r="AG77" s="25"/>
-      <c r="AH77" s="61"/>
+      <c r="AF77" s="25"/>
+      <c r="AG77" s="61"/>
+      <c r="AH77" s="42"/>
       <c r="AI77" s="42"/>
-      <c r="AJ77" s="42"/>
-      <c r="AK77" s="39"/>
-    </row>
-    <row r="78" spans="1:37" ht="48" customHeight="1">
+      <c r="AJ77" s="39"/>
+    </row>
+    <row r="78" spans="1:36" ht="48" customHeight="1">
       <c r="A78" s="61"/>
       <c r="B78" s="42"/>
       <c r="C78" s="42"/>
@@ -10179,14 +10077,13 @@
       <c r="AC78" s="65"/>
       <c r="AD78" s="65"/>
       <c r="AE78" s="65"/>
-      <c r="AF78" s="65"/>
-      <c r="AG78" s="25"/>
+      <c r="AF78" s="25"/>
+      <c r="AG78" s="42"/>
       <c r="AH78" s="42"/>
       <c r="AI78" s="42"/>
-      <c r="AJ78" s="42"/>
-      <c r="AK78" s="39"/>
-    </row>
-    <row r="79" spans="1:37">
+      <c r="AJ78" s="39"/>
+    </row>
+    <row r="79" spans="1:36">
       <c r="A79" s="61"/>
       <c r="B79" s="42"/>
       <c r="C79" s="61"/>
@@ -10221,14 +10118,13 @@
       <c r="AC79" s="65"/>
       <c r="AD79" s="65"/>
       <c r="AE79" s="65"/>
-      <c r="AF79" s="65"/>
-      <c r="AG79" s="59"/>
+      <c r="AF79" s="59"/>
+      <c r="AG79" s="61"/>
       <c r="AH79" s="61"/>
-      <c r="AI79" s="61"/>
-      <c r="AJ79" s="42"/>
-      <c r="AK79" s="39"/>
-    </row>
-    <row r="80" spans="1:37">
+      <c r="AI79" s="42"/>
+      <c r="AJ79" s="39"/>
+    </row>
+    <row r="80" spans="1:36">
       <c r="A80" s="61"/>
       <c r="B80" s="62"/>
       <c r="C80" s="61"/>
@@ -10263,14 +10159,13 @@
       <c r="AC80" s="65"/>
       <c r="AD80" s="65"/>
       <c r="AE80" s="65"/>
-      <c r="AF80" s="65"/>
-      <c r="AG80" s="59"/>
-      <c r="AH80" s="62"/>
-      <c r="AI80" s="61"/>
-      <c r="AJ80" s="42"/>
-      <c r="AK80" s="39"/>
-    </row>
-    <row r="81" spans="1:37">
+      <c r="AF80" s="59"/>
+      <c r="AG80" s="62"/>
+      <c r="AH80" s="61"/>
+      <c r="AI80" s="42"/>
+      <c r="AJ80" s="39"/>
+    </row>
+    <row r="81" spans="1:36">
       <c r="A81" s="61"/>
       <c r="B81" s="61"/>
       <c r="C81" s="61"/>
@@ -10305,14 +10200,13 @@
       <c r="AC81" s="65"/>
       <c r="AD81" s="65"/>
       <c r="AE81" s="65"/>
-      <c r="AF81" s="65"/>
-      <c r="AG81" s="59"/>
+      <c r="AF81" s="59"/>
+      <c r="AG81" s="61"/>
       <c r="AH81" s="61"/>
-      <c r="AI81" s="61"/>
-      <c r="AJ81" s="42"/>
-      <c r="AK81" s="39"/>
-    </row>
-    <row r="82" spans="1:37">
+      <c r="AI81" s="42"/>
+      <c r="AJ81" s="39"/>
+    </row>
+    <row r="82" spans="1:36">
       <c r="A82" s="61"/>
       <c r="B82" s="61"/>
       <c r="C82" s="61"/>
@@ -10347,14 +10241,13 @@
       <c r="AC82" s="65"/>
       <c r="AD82" s="65"/>
       <c r="AE82" s="65"/>
-      <c r="AF82" s="65"/>
-      <c r="AG82" s="59"/>
+      <c r="AF82" s="59"/>
+      <c r="AG82" s="61"/>
       <c r="AH82" s="61"/>
-      <c r="AI82" s="61"/>
-      <c r="AJ82" s="42"/>
-      <c r="AK82" s="39"/>
-    </row>
-    <row r="83" spans="1:37">
+      <c r="AI82" s="42"/>
+      <c r="AJ82" s="39"/>
+    </row>
+    <row r="83" spans="1:36">
       <c r="A83" s="61"/>
       <c r="B83" s="61"/>
       <c r="C83" s="61"/>
@@ -10375,13 +10268,13 @@
       <c r="O83" s="8"/>
       <c r="P83" s="8"/>
       <c r="Q83" s="65"/>
-      <c r="R83" s="65"/>
+      <c r="R83" s="8"/>
       <c r="S83" s="8"/>
       <c r="T83" s="8"/>
       <c r="U83" s="8"/>
       <c r="V83" s="8"/>
       <c r="W83" s="8"/>
-      <c r="X83" s="8"/>
+      <c r="X83" s="65"/>
       <c r="Y83" s="65"/>
       <c r="Z83" s="65"/>
       <c r="AA83" s="65"/>
@@ -10389,14 +10282,13 @@
       <c r="AC83" s="65"/>
       <c r="AD83" s="65"/>
       <c r="AE83" s="65"/>
-      <c r="AF83" s="65"/>
-      <c r="AG83" s="59"/>
-      <c r="AH83" s="42"/>
-      <c r="AI83" s="66"/>
-      <c r="AJ83" s="42"/>
-      <c r="AK83" s="39"/>
-    </row>
-    <row r="84" spans="1:37">
+      <c r="AF83" s="59"/>
+      <c r="AG83" s="42"/>
+      <c r="AH83" s="66"/>
+      <c r="AI83" s="42"/>
+      <c r="AJ83" s="39"/>
+    </row>
+    <row r="84" spans="1:36">
       <c r="A84" s="61"/>
       <c r="B84" s="6"/>
       <c r="C84" s="6"/>
@@ -10417,10 +10309,10 @@
       <c r="O84" s="8"/>
       <c r="P84" s="8"/>
       <c r="Q84" s="8"/>
-      <c r="R84" s="8"/>
+      <c r="R84" s="53"/>
       <c r="S84" s="53"/>
       <c r="T84" s="53"/>
-      <c r="U84" s="53"/>
+      <c r="U84" s="8"/>
       <c r="V84" s="8"/>
       <c r="W84" s="8"/>
       <c r="X84" s="8"/>
@@ -10431,14 +10323,13 @@
       <c r="AC84" s="8"/>
       <c r="AD84" s="8"/>
       <c r="AE84" s="8"/>
-      <c r="AF84" s="8"/>
-      <c r="AG84" s="25"/>
-      <c r="AH84" s="6"/>
-      <c r="AI84" s="63"/>
-      <c r="AJ84" s="42"/>
-      <c r="AK84" s="39"/>
-    </row>
-    <row r="85" spans="1:37">
+      <c r="AF84" s="25"/>
+      <c r="AG84" s="6"/>
+      <c r="AH84" s="63"/>
+      <c r="AI84" s="42"/>
+      <c r="AJ84" s="39"/>
+    </row>
+    <row r="85" spans="1:36">
       <c r="A85" s="61"/>
       <c r="B85" s="61"/>
       <c r="C85" s="61"/>
@@ -10459,13 +10350,13 @@
       <c r="O85" s="8"/>
       <c r="P85" s="8"/>
       <c r="Q85" s="8"/>
-      <c r="R85" s="8"/>
+      <c r="R85" s="53"/>
       <c r="S85" s="53"/>
       <c r="T85" s="53"/>
-      <c r="U85" s="53"/>
+      <c r="U85" s="8"/>
       <c r="V85" s="8"/>
       <c r="W85" s="8"/>
-      <c r="X85" s="8"/>
+      <c r="X85" s="65"/>
       <c r="Y85" s="65"/>
       <c r="Z85" s="65"/>
       <c r="AA85" s="65"/>
@@ -10473,14 +10364,13 @@
       <c r="AC85" s="65"/>
       <c r="AD85" s="65"/>
       <c r="AE85" s="65"/>
-      <c r="AF85" s="65"/>
-      <c r="AG85" s="59"/>
+      <c r="AF85" s="59"/>
+      <c r="AG85" s="61"/>
       <c r="AH85" s="61"/>
-      <c r="AI85" s="61"/>
-      <c r="AJ85" s="42"/>
-      <c r="AK85" s="39"/>
-    </row>
-    <row r="86" spans="1:37">
+      <c r="AI85" s="42"/>
+      <c r="AJ85" s="39"/>
+    </row>
+    <row r="86" spans="1:36">
       <c r="A86" s="61"/>
       <c r="B86" s="61"/>
       <c r="C86" s="61"/>
@@ -10501,13 +10391,13 @@
       <c r="O86" s="8"/>
       <c r="P86" s="8"/>
       <c r="Q86" s="8"/>
-      <c r="R86" s="8"/>
+      <c r="R86" s="53"/>
       <c r="S86" s="53"/>
       <c r="T86" s="53"/>
-      <c r="U86" s="53"/>
+      <c r="U86" s="8"/>
       <c r="V86" s="8"/>
       <c r="W86" s="8"/>
-      <c r="X86" s="8"/>
+      <c r="X86" s="65"/>
       <c r="Y86" s="65"/>
       <c r="Z86" s="65"/>
       <c r="AA86" s="65"/>
@@ -10515,14 +10405,13 @@
       <c r="AC86" s="65"/>
       <c r="AD86" s="65"/>
       <c r="AE86" s="65"/>
-      <c r="AF86" s="65"/>
-      <c r="AG86" s="59"/>
+      <c r="AF86" s="59"/>
+      <c r="AG86" s="61"/>
       <c r="AH86" s="61"/>
-      <c r="AI86" s="61"/>
-      <c r="AJ86" s="42"/>
-      <c r="AK86" s="39"/>
-    </row>
-    <row r="87" spans="1:37">
+      <c r="AI86" s="42"/>
+      <c r="AJ86" s="39"/>
+    </row>
+    <row r="87" spans="1:36">
       <c r="A87" s="42"/>
       <c r="B87" s="61"/>
       <c r="C87" s="61"/>
@@ -10549,7 +10438,7 @@
       <c r="U87" s="8"/>
       <c r="V87" s="8"/>
       <c r="W87" s="8"/>
-      <c r="X87" s="8"/>
+      <c r="X87" s="65"/>
       <c r="Y87" s="65"/>
       <c r="Z87" s="65"/>
       <c r="AA87" s="65"/>
@@ -10557,14 +10446,13 @@
       <c r="AC87" s="65"/>
       <c r="AD87" s="65"/>
       <c r="AE87" s="65"/>
-      <c r="AF87" s="65"/>
-      <c r="AG87" s="59"/>
+      <c r="AF87" s="59"/>
+      <c r="AG87" s="61"/>
       <c r="AH87" s="61"/>
-      <c r="AI87" s="61"/>
-      <c r="AJ87" s="42"/>
-      <c r="AK87" s="39"/>
-    </row>
-    <row r="88" spans="1:37">
+      <c r="AI87" s="42"/>
+      <c r="AJ87" s="39"/>
+    </row>
+    <row r="88" spans="1:36">
       <c r="A88" s="42"/>
       <c r="B88" s="6"/>
       <c r="C88" s="6"/>
@@ -10585,10 +10473,10 @@
       <c r="O88" s="8"/>
       <c r="P88" s="8"/>
       <c r="Q88" s="8"/>
-      <c r="R88" s="8"/>
+      <c r="R88" s="53"/>
       <c r="S88" s="53"/>
       <c r="T88" s="53"/>
-      <c r="U88" s="53"/>
+      <c r="U88" s="8"/>
       <c r="V88" s="8"/>
       <c r="W88" s="8"/>
       <c r="X88" s="8"/>
@@ -10599,14 +10487,13 @@
       <c r="AC88" s="8"/>
       <c r="AD88" s="8"/>
       <c r="AE88" s="8"/>
-      <c r="AF88" s="8"/>
-      <c r="AG88" s="25"/>
-      <c r="AH88" s="6"/>
-      <c r="AI88" s="63"/>
-      <c r="AJ88" s="42"/>
-      <c r="AK88" s="39"/>
-    </row>
-    <row r="89" spans="1:37">
+      <c r="AF88" s="25"/>
+      <c r="AG88" s="6"/>
+      <c r="AH88" s="63"/>
+      <c r="AI88" s="42"/>
+      <c r="AJ88" s="39"/>
+    </row>
+    <row r="89" spans="1:36">
       <c r="A89" s="42"/>
       <c r="B89" s="42"/>
       <c r="C89" s="42"/>
@@ -10627,13 +10514,13 @@
       <c r="O89" s="8"/>
       <c r="P89" s="8"/>
       <c r="Q89" s="8"/>
-      <c r="R89" s="8"/>
+      <c r="R89" s="53"/>
       <c r="S89" s="53"/>
-      <c r="T89" s="53"/>
+      <c r="T89" s="8"/>
       <c r="U89" s="8"/>
       <c r="V89" s="8"/>
       <c r="W89" s="8"/>
-      <c r="X89" s="8"/>
+      <c r="X89" s="39"/>
       <c r="Y89" s="39"/>
       <c r="Z89" s="39"/>
       <c r="AA89" s="39"/>
@@ -10641,14 +10528,13 @@
       <c r="AC89" s="39"/>
       <c r="AD89" s="39"/>
       <c r="AE89" s="39"/>
-      <c r="AF89" s="39"/>
-      <c r="AG89" s="48"/>
-      <c r="AH89" s="42"/>
-      <c r="AI89" s="6"/>
-      <c r="AJ89" s="42"/>
-      <c r="AK89" s="39"/>
-    </row>
-    <row r="90" spans="1:37">
+      <c r="AF89" s="48"/>
+      <c r="AG89" s="42"/>
+      <c r="AH89" s="6"/>
+      <c r="AI89" s="42"/>
+      <c r="AJ89" s="39"/>
+    </row>
+    <row r="90" spans="1:36">
       <c r="A90" s="42"/>
       <c r="B90" s="42"/>
       <c r="C90" s="6"/>
@@ -10669,10 +10555,10 @@
       <c r="O90" s="8"/>
       <c r="P90" s="8"/>
       <c r="Q90" s="8"/>
-      <c r="R90" s="8"/>
-      <c r="S90" s="42"/>
-      <c r="T90" s="53"/>
-      <c r="U90" s="42"/>
+      <c r="R90" s="42"/>
+      <c r="S90" s="53"/>
+      <c r="T90" s="42"/>
+      <c r="U90" s="8"/>
       <c r="V90" s="8"/>
       <c r="W90" s="8"/>
       <c r="X90" s="8"/>
@@ -10683,12 +10569,11 @@
       <c r="AC90" s="8"/>
       <c r="AD90" s="8"/>
       <c r="AE90" s="8"/>
-      <c r="AF90" s="8"/>
-      <c r="AG90" s="25"/>
+      <c r="AF90" s="25"/>
+      <c r="AG90" s="42"/>
       <c r="AH90" s="42"/>
       <c r="AI90" s="42"/>
-      <c r="AJ90" s="42"/>
-      <c r="AK90" s="39"/>
+      <c r="AJ90" s="39"/>
     </row>
   </sheetData>
   <dataValidations count="4">
@@ -10698,7 +10583,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P6:P90" xr:uid="{00000000-0002-0000-0700-000001000000}">
       <formula1>"unidirectional,bidirectional"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V6:V90 E6:E90 G84:G90 F6:F17 F19 F21:F22 F24:F31 H6:M90 G6:G33 F33:F49 G35:G51 F51:F57 G53:G59 F59:F76 G61:G78 F78:F79 G80:G81 F81:F83 F85:F90" xr:uid="{00000000-0002-0000-0700-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U6:U90 E6:E90 G84:G90 F6:F17 F19 F21:F22 F24:F31 H6:M90 G6:G33 F33:F49 G35:G51 F51:F57 G53:G59 F59:F76 G61:G78 F78:F79 G80:G81 F81:F83 F85:F90" xr:uid="{00000000-0002-0000-0700-000002000000}">
       <formula1>"○"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N6:N90" xr:uid="{00000000-0002-0000-0700-000003000000}">
@@ -10715,7 +10600,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:AK90"/>
+  <dimension ref="A1:AJ90"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="39.1640625" style="35" bestFit="1" customWidth="1"/>
@@ -10732,60 +10617,59 @@
     <col min="14" max="14" width="8.5" style="37" customWidth="1" outlineLevel="1"/>
     <col min="15" max="16" width="18.33203125" style="37" customWidth="1" outlineLevel="2"/>
     <col min="17" max="17" width="29.5" style="37" customWidth="1" outlineLevel="2"/>
-    <col min="18" max="18" width="24.33203125" style="37" customWidth="1" outlineLevel="2"/>
-    <col min="19" max="19" width="29" style="37" customWidth="1" outlineLevel="2"/>
-    <col min="20" max="21" width="18.33203125" style="37" customWidth="1" outlineLevel="2"/>
-    <col min="22" max="22" width="17.1640625" style="37" bestFit="1" customWidth="1" outlineLevel="1"/>
-    <col min="23" max="24" width="9.1640625" style="37" hidden="1" customWidth="1" outlineLevel="2"/>
-    <col min="25" max="25" width="9.33203125" style="37" hidden="1" customWidth="1" outlineLevel="2"/>
-    <col min="26" max="26" width="37.5" style="35" hidden="1" customWidth="1" outlineLevel="2"/>
-    <col min="27" max="32" width="19.33203125" style="38" hidden="1" customWidth="1" outlineLevel="2"/>
-    <col min="33" max="33" width="19.33203125" style="38" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <col min="34" max="37" width="19.33203125" style="38" customWidth="1"/>
+    <col min="18" max="18" width="29" style="37" customWidth="1" outlineLevel="2"/>
+    <col min="19" max="20" width="18.33203125" style="37" customWidth="1" outlineLevel="2"/>
+    <col min="21" max="21" width="17.1640625" style="37" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="22" max="23" width="9.1640625" style="37" hidden="1" customWidth="1" outlineLevel="2"/>
+    <col min="24" max="24" width="9.33203125" style="37" hidden="1" customWidth="1" outlineLevel="2"/>
+    <col min="25" max="25" width="37.5" style="35" hidden="1" customWidth="1" outlineLevel="2"/>
+    <col min="26" max="31" width="19.33203125" style="38" hidden="1" customWidth="1" outlineLevel="2"/>
+    <col min="32" max="32" width="19.33203125" style="38" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <col min="33" max="36" width="19.33203125" style="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37">
+    <row r="1" spans="1:36">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:37" ht="16" customHeight="1">
+    <row r="2" spans="1:36" ht="16" customHeight="1">
+      <c r="AG2" s="71" t="s">
+        <v>1</v>
+      </c>
       <c r="AH2" s="71" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI2" s="71" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AJ2" s="71" t="s">
-        <v>3</v>
-      </c>
-      <c r="AK2" s="71" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:37">
+    <row r="3" spans="1:36">
       <c r="A3" s="52"/>
-      <c r="AH3" s="32" t="str">
+      <c r="AG3" s="32" t="str">
         <f>IF('General Settings'!$G$11=0,"",'General Settings'!$G$11)</f>
         <v>en</v>
       </c>
+      <c r="AH3" s="32" t="str">
+        <f>IF('General Settings'!$G$12=0,"",'General Settings'!$G$12)</f>
+        <v/>
+      </c>
       <c r="AI3" s="32" t="str">
-        <f>IF('General Settings'!$G$12=0,"",'General Settings'!$G$12)</f>
+        <f>IF('General Settings'!$G$13=0,"",'General Settings'!$G$13)</f>
         <v/>
       </c>
       <c r="AJ3" s="32" t="str">
-        <f>IF('General Settings'!$G$13=0,"",'General Settings'!$G$13)</f>
-        <v/>
-      </c>
-      <c r="AK3" s="32" t="str">
         <f>IF('General Settings'!$G$14=0,"",'General Settings'!$G$14)</f>
         <v/>
       </c>
     </row>
-    <row r="4" spans="1:37">
+    <row r="4" spans="1:36">
       <c r="A4" s="34"/>
     </row>
-    <row r="5" spans="1:37" s="1" customFormat="1" ht="43" customHeight="1">
+    <row r="5" spans="1:36" s="1" customFormat="1" ht="43" customHeight="1">
       <c r="A5" s="101" t="s">
         <v>5</v>
       </c>
@@ -10849,7 +10733,7 @@
       <c r="U5" s="74" t="s">
         <v>25</v>
       </c>
-      <c r="V5" s="74" t="s">
+      <c r="V5" s="107" t="s">
         <v>26</v>
       </c>
       <c r="W5" s="107" t="s">
@@ -10879,13 +10763,13 @@
       <c r="AE5" s="107" t="s">
         <v>35</v>
       </c>
-      <c r="AF5" s="107" t="s">
+      <c r="AF5" s="74" t="s">
         <v>36</v>
       </c>
-      <c r="AG5" s="74" t="s">
+      <c r="AG5" s="73" t="s">
         <v>37</v>
       </c>
-      <c r="AH5" s="73" t="s">
+      <c r="AH5" s="75" t="s">
         <v>38</v>
       </c>
       <c r="AI5" s="75" t="s">
@@ -10894,11 +10778,8 @@
       <c r="AJ5" s="75" t="s">
         <v>40</v>
       </c>
-      <c r="AK5" s="75" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:37" s="1" customFormat="1">
+    </row>
+    <row r="6" spans="1:36" s="1" customFormat="1">
       <c r="A6" s="79"/>
       <c r="B6" s="81"/>
       <c r="C6" s="80"/>
@@ -10919,11 +10800,11 @@
       <c r="O6" s="87"/>
       <c r="P6" s="87"/>
       <c r="Q6" s="87"/>
-      <c r="R6" s="87"/>
+      <c r="R6" s="85"/>
       <c r="S6" s="85"/>
-      <c r="T6" s="85"/>
-      <c r="U6" s="57"/>
-      <c r="V6" s="91"/>
+      <c r="T6" s="57"/>
+      <c r="U6" s="91"/>
+      <c r="V6" s="90"/>
       <c r="W6" s="90"/>
       <c r="X6" s="90"/>
       <c r="Y6" s="90"/>
@@ -10933,14 +10814,13 @@
       <c r="AC6" s="90"/>
       <c r="AD6" s="90"/>
       <c r="AE6" s="90"/>
-      <c r="AF6" s="90"/>
-      <c r="AG6" s="102"/>
-      <c r="AH6" s="80"/>
-      <c r="AI6" s="54"/>
-      <c r="AJ6" s="42"/>
-      <c r="AK6" s="39"/>
-    </row>
-    <row r="7" spans="1:37" s="1" customFormat="1">
+      <c r="AF6" s="102"/>
+      <c r="AG6" s="80"/>
+      <c r="AH6" s="54"/>
+      <c r="AI6" s="42"/>
+      <c r="AJ6" s="39"/>
+    </row>
+    <row r="7" spans="1:36" s="1" customFormat="1">
       <c r="A7" s="88"/>
       <c r="B7" s="90"/>
       <c r="C7" s="89"/>
@@ -10961,11 +10841,11 @@
       <c r="O7" s="47"/>
       <c r="P7" s="47"/>
       <c r="Q7" s="47"/>
-      <c r="R7" s="47"/>
+      <c r="R7" s="57"/>
       <c r="S7" s="57"/>
       <c r="T7" s="57"/>
-      <c r="U7" s="57"/>
-      <c r="V7" s="91"/>
+      <c r="U7" s="91"/>
+      <c r="V7" s="57"/>
       <c r="W7" s="57"/>
       <c r="X7" s="57"/>
       <c r="Y7" s="57"/>
@@ -10975,14 +10855,13 @@
       <c r="AC7" s="57"/>
       <c r="AD7" s="57"/>
       <c r="AE7" s="57"/>
-      <c r="AF7" s="57"/>
-      <c r="AG7" s="103"/>
-      <c r="AH7" s="89"/>
-      <c r="AI7" s="54"/>
-      <c r="AJ7" s="42"/>
-      <c r="AK7" s="39"/>
-    </row>
-    <row r="8" spans="1:37" s="1" customFormat="1">
+      <c r="AF7" s="103"/>
+      <c r="AG7" s="89"/>
+      <c r="AH7" s="54"/>
+      <c r="AI7" s="42"/>
+      <c r="AJ7" s="39"/>
+    </row>
+    <row r="8" spans="1:36" s="1" customFormat="1">
       <c r="A8" s="79"/>
       <c r="B8" s="81"/>
       <c r="C8" s="93"/>
@@ -11003,11 +10882,11 @@
       <c r="O8" s="87"/>
       <c r="P8" s="87"/>
       <c r="Q8" s="87"/>
-      <c r="R8" s="87"/>
+      <c r="R8" s="94"/>
       <c r="S8" s="94"/>
-      <c r="T8" s="94"/>
-      <c r="U8" s="104"/>
-      <c r="V8" s="91"/>
+      <c r="T8" s="104"/>
+      <c r="U8" s="91"/>
+      <c r="V8" s="99"/>
       <c r="W8" s="99"/>
       <c r="X8" s="99"/>
       <c r="Y8" s="99"/>
@@ -11017,14 +10896,13 @@
       <c r="AC8" s="99"/>
       <c r="AD8" s="99"/>
       <c r="AE8" s="99"/>
-      <c r="AF8" s="99"/>
-      <c r="AG8" s="105"/>
-      <c r="AH8" s="80"/>
-      <c r="AI8" s="54"/>
-      <c r="AJ8" s="42"/>
-      <c r="AK8" s="39"/>
-    </row>
-    <row r="9" spans="1:37">
+      <c r="AF8" s="105"/>
+      <c r="AG8" s="80"/>
+      <c r="AH8" s="54"/>
+      <c r="AI8" s="42"/>
+      <c r="AJ8" s="39"/>
+    </row>
+    <row r="9" spans="1:36">
       <c r="A9" s="88"/>
       <c r="B9" s="97"/>
       <c r="C9" s="89"/>
@@ -11048,8 +10926,8 @@
       <c r="R9" s="47"/>
       <c r="S9" s="47"/>
       <c r="T9" s="47"/>
-      <c r="U9" s="47"/>
-      <c r="V9" s="91"/>
+      <c r="U9" s="91"/>
+      <c r="V9" s="47"/>
       <c r="W9" s="47"/>
       <c r="X9" s="47"/>
       <c r="Y9" s="47"/>
@@ -11059,14 +10937,13 @@
       <c r="AC9" s="47"/>
       <c r="AD9" s="47"/>
       <c r="AE9" s="47"/>
-      <c r="AF9" s="47"/>
-      <c r="AG9" s="106"/>
-      <c r="AH9" s="96"/>
-      <c r="AI9" s="120"/>
-      <c r="AJ9" s="42"/>
-      <c r="AK9" s="39"/>
-    </row>
-    <row r="10" spans="1:37">
+      <c r="AF9" s="106"/>
+      <c r="AG9" s="96"/>
+      <c r="AH9" s="120"/>
+      <c r="AI9" s="42"/>
+      <c r="AJ9" s="39"/>
+    </row>
+    <row r="10" spans="1:36">
       <c r="A10" s="79"/>
       <c r="B10" s="100"/>
       <c r="C10" s="80"/>
@@ -11089,9 +10966,9 @@
       <c r="Q10" s="87"/>
       <c r="R10" s="87"/>
       <c r="S10" s="87"/>
-      <c r="T10" s="87"/>
-      <c r="U10" s="47"/>
-      <c r="V10" s="91"/>
+      <c r="T10" s="47"/>
+      <c r="U10" s="91"/>
+      <c r="V10" s="47"/>
       <c r="W10" s="47"/>
       <c r="X10" s="47"/>
       <c r="Y10" s="47"/>
@@ -11101,14 +10978,13 @@
       <c r="AC10" s="47"/>
       <c r="AD10" s="47"/>
       <c r="AE10" s="47"/>
-      <c r="AF10" s="47"/>
-      <c r="AG10" s="106"/>
-      <c r="AH10" s="93"/>
-      <c r="AI10" s="120"/>
-      <c r="AJ10" s="42"/>
-      <c r="AK10" s="39"/>
-    </row>
-    <row r="11" spans="1:37">
+      <c r="AF10" s="106"/>
+      <c r="AG10" s="93"/>
+      <c r="AH10" s="120"/>
+      <c r="AI10" s="42"/>
+      <c r="AJ10" s="39"/>
+    </row>
+    <row r="11" spans="1:36">
       <c r="A11" s="88"/>
       <c r="B11" s="96"/>
       <c r="C11" s="96"/>
@@ -11132,8 +11008,8 @@
       <c r="R11" s="47"/>
       <c r="S11" s="47"/>
       <c r="T11" s="47"/>
-      <c r="U11" s="47"/>
-      <c r="V11" s="91"/>
+      <c r="U11" s="91"/>
+      <c r="V11" s="47"/>
       <c r="W11" s="47"/>
       <c r="X11" s="47"/>
       <c r="Y11" s="47"/>
@@ -11143,14 +11019,13 @@
       <c r="AC11" s="47"/>
       <c r="AD11" s="47"/>
       <c r="AE11" s="47"/>
-      <c r="AF11" s="47"/>
-      <c r="AG11" s="106"/>
-      <c r="AH11" s="96"/>
-      <c r="AI11" s="120"/>
-      <c r="AJ11" s="42"/>
-      <c r="AK11" s="39"/>
-    </row>
-    <row r="12" spans="1:37">
+      <c r="AF11" s="106"/>
+      <c r="AG11" s="96"/>
+      <c r="AH11" s="120"/>
+      <c r="AI11" s="42"/>
+      <c r="AJ11" s="39"/>
+    </row>
+    <row r="12" spans="1:36">
       <c r="A12" s="79"/>
       <c r="B12" s="93"/>
       <c r="C12" s="93"/>
@@ -11173,9 +11048,9 @@
       <c r="Q12" s="87"/>
       <c r="R12" s="87"/>
       <c r="S12" s="87"/>
-      <c r="T12" s="87"/>
-      <c r="U12" s="47"/>
-      <c r="V12" s="91"/>
+      <c r="T12" s="47"/>
+      <c r="U12" s="91"/>
+      <c r="V12" s="47"/>
       <c r="W12" s="47"/>
       <c r="X12" s="47"/>
       <c r="Y12" s="47"/>
@@ -11185,14 +11060,13 @@
       <c r="AC12" s="47"/>
       <c r="AD12" s="47"/>
       <c r="AE12" s="47"/>
-      <c r="AF12" s="47"/>
-      <c r="AG12" s="106"/>
-      <c r="AH12" s="93"/>
-      <c r="AI12" s="120"/>
-      <c r="AJ12" s="42"/>
-      <c r="AK12" s="39"/>
-    </row>
-    <row r="13" spans="1:37">
+      <c r="AF12" s="106"/>
+      <c r="AG12" s="93"/>
+      <c r="AH12" s="120"/>
+      <c r="AI12" s="42"/>
+      <c r="AJ12" s="39"/>
+    </row>
+    <row r="13" spans="1:36">
       <c r="A13" s="88"/>
       <c r="B13" s="96"/>
       <c r="C13" s="96"/>
@@ -11216,8 +11090,8 @@
       <c r="R13" s="47"/>
       <c r="S13" s="47"/>
       <c r="T13" s="47"/>
-      <c r="U13" s="47"/>
-      <c r="V13" s="91"/>
+      <c r="U13" s="91"/>
+      <c r="V13" s="47"/>
       <c r="W13" s="47"/>
       <c r="X13" s="47"/>
       <c r="Y13" s="47"/>
@@ -11227,20 +11101,19 @@
       <c r="AC13" s="47"/>
       <c r="AD13" s="47"/>
       <c r="AE13" s="47"/>
-      <c r="AF13" s="47"/>
-      <c r="AG13" s="106"/>
-      <c r="AH13" s="96"/>
-      <c r="AI13" s="51"/>
-      <c r="AJ13" s="42"/>
-      <c r="AK13" s="39"/>
-    </row>
-    <row r="14" spans="1:37">
+      <c r="AF13" s="106"/>
+      <c r="AG13" s="96"/>
+      <c r="AH13" s="51"/>
+      <c r="AI13" s="42"/>
+      <c r="AJ13" s="39"/>
+    </row>
+    <row r="14" spans="1:36">
       <c r="H14" s="8"/>
     </row>
-    <row r="15" spans="1:37">
+    <row r="15" spans="1:36">
       <c r="H15" s="8"/>
     </row>
-    <row r="16" spans="1:37">
+    <row r="16" spans="1:36">
       <c r="H16" s="8"/>
     </row>
     <row r="17" spans="8:8">
@@ -11281,12 +11154,12 @@
     </row>
     <row r="29" spans="8:8">
       <c r="H29" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="30" spans="8:8">
       <c r="H30" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="31" spans="8:8">
@@ -11306,22 +11179,22 @@
     </row>
     <row r="36" spans="8:8">
       <c r="H36" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="37" spans="8:8">
       <c r="H37" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="38" spans="8:8">
       <c r="H38" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="39" spans="8:8">
       <c r="H39" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="40" spans="8:8">
@@ -11335,32 +11208,32 @@
     </row>
     <row r="43" spans="8:8">
       <c r="H43" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="44" spans="8:8">
       <c r="H44" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="45" spans="8:8">
       <c r="H45" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="46" spans="8:8">
       <c r="H46" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="47" spans="8:8">
       <c r="H47" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="48" spans="8:8">
       <c r="H48" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="49" spans="8:8">
@@ -11380,7 +11253,7 @@
     </row>
     <row r="54" spans="8:8">
       <c r="H54" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="55" spans="8:8">
@@ -11412,7 +11285,7 @@
     </row>
     <row r="64" spans="8:8">
       <c r="H64" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="65" spans="8:8">
@@ -11441,17 +11314,17 @@
     </row>
     <row r="73" spans="8:8">
       <c r="H73" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="74" spans="8:8">
       <c r="H74" s="65" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="75" spans="8:8">
       <c r="H75" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="76" spans="8:8">
@@ -11489,7 +11362,7 @@
     </row>
     <row r="87" spans="8:8">
       <c r="H87" s="65" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="88" spans="8:8">
@@ -11506,7 +11379,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N6:N13" xr:uid="{00000000-0002-0000-0800-000000000000}">
       <formula1>"CB,CD,LB,LD"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V6:V13 E6:E13 F6:G13 I6:M13 H6:H90" xr:uid="{00000000-0002-0000-0800-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U6:U13 E6:E13 F6:G13 I6:M13 H6:H90" xr:uid="{00000000-0002-0000-0800-000001000000}">
       <formula1>"○"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O6:O13" xr:uid="{00000000-0002-0000-0800-000002000000}">

</xml_diff>

<commit_message>
DataType Definition: sheet name fixed in English excel-format
</commit_message>
<xml_diff>
--- a/excel-format/db-column-definitions_fmt-v5.0.0-en_my-app.xlsx
+++ b/excel-format/db-column-definitions_fmt-v5.0.0-en_my-app.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yosuke.tanaka/Desktop/development/git/ecuacion-tool-code-generator/excel-format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85311384-5ABC-1A4E-996E-CB96299EFD65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58D1ECD4-4030-0240-B7F1-0713BB94DEFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17500" tabRatio="853" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="FK Types" sheetId="3" state="hidden" r:id="rId3"/>
     <sheet name="Format Change History" sheetId="4" r:id="rId4"/>
     <sheet name="General Settings" sheetId="5" r:id="rId5"/>
-    <sheet name="dataType Definition" sheetId="6" r:id="rId6"/>
+    <sheet name="DataType Definition" sheetId="6" r:id="rId6"/>
     <sheet name="Enum Definition" sheetId="7" r:id="rId7"/>
     <sheet name="DB Item Definition" sheetId="8" r:id="rId8"/>
     <sheet name="DB Common Item Definition" sheetId="9" r:id="rId9"/>
@@ -128,7 +128,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="220">
   <si>
     <t>DB Common Item Definition</t>
   </si>
@@ -811,6 +811,9 @@
   </si>
   <si>
     <t>For Binary</t>
+  </si>
+  <si>
+    <t>DataType Definition</t>
   </si>
 </sst>
 </file>
@@ -1448,35 +1451,31 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="標準 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="126">
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="center"/>
@@ -2710,6 +2709,93 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.34998626667073579"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
@@ -2805,6 +2891,10 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -2814,93 +2904,6 @@
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -3010,114 +3013,114 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table5" displayName="Table5" ref="A3:D4" totalsRowShown="0" headerRowDxfId="125" dataDxfId="124">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table5" displayName="Table5" ref="A3:D4" totalsRowShown="0" headerRowDxfId="104" dataDxfId="103">
   <autoFilter ref="A3:D4" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Date" dataDxfId="123"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Version" dataDxfId="122"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Changes" dataDxfId="121"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Changed By" dataDxfId="120"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Date" dataDxfId="102"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Version" dataDxfId="101"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Changes" dataDxfId="100"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Changed By" dataDxfId="99"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table50" displayName="Table50" ref="A5:H28" totalsRowShown="0" dataDxfId="119">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table50" displayName="Table50" ref="A5:H28" totalsRowShown="0" dataDxfId="98">
   <autoFilter ref="A5:H28" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="#" dataDxfId="118">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="#" dataDxfId="97">
       <calculatedColumnFormula>ROW()-5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="Category" dataDxfId="117"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Category Name" dataDxfId="116"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Key" dataDxfId="115"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Description" dataDxfId="114"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="Required" dataDxfId="113"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Value" dataDxfId="112"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Notes" dataDxfId="111"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="Category" dataDxfId="96"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Category Name" dataDxfId="95"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Key" dataDxfId="94"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Description" dataDxfId="93"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="Required" dataDxfId="92"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Value" dataDxfId="91"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Notes" dataDxfId="90"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table2" displayName="Table2" ref="A7:T10" tableType="xml" totalsRowShown="0" headerRowDxfId="110" dataDxfId="109">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table2" displayName="Table2" ref="A7:T10" tableType="xml" totalsRowShown="0" headerRowDxfId="125" dataDxfId="124">
   <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" uniqueName="name" name="DataType Name" dataDxfId="108">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" uniqueName="name" name="DataType Name" dataDxfId="123">
       <xmlColumnPr mapId="191" xpath="/root/datatype/@name" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" uniqueName="kata" name="Type" dataDxfId="0">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" uniqueName="kata" name="Type" dataDxfId="122">
       <xmlColumnPr mapId="191" xpath="/root/datatype/kata" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" uniqueName="minLength" name="Min Length" dataDxfId="107">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" uniqueName="minLength" name="Min Length" dataDxfId="121">
       <xmlColumnPr mapId="191" xpath="/root/datatype/minLength" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0400-00000B000000}" uniqueName="maxLength" name="Max Length" dataDxfId="106">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0400-00000B000000}" uniqueName="maxLength" name="Max Length" dataDxfId="120">
       <xmlColumnPr mapId="191" xpath="/root/datatype/maxLength" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0400-00000F000000}" uniqueName="numScale" name="Data Pattern (display name)" dataDxfId="105"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0400-000018000000}" uniqueName="stringDataPtn" name="Data Pattern" dataDxfId="104">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0400-00000F000000}" uniqueName="numScale" name="Data Pattern (display name)" dataDxfId="119"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0400-000018000000}" uniqueName="stringDataPtn" name="Data Pattern" dataDxfId="118">
       <xmlColumnPr mapId="191" xpath="/root/datatype/stringDataPtn" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0400-000012000000}" uniqueName="18" name="Exclude Prohibited Chars Check" dataDxfId="103"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0400-000019000000}" uniqueName="stringRegEx" name="Regex" dataDxfId="102">
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0400-000012000000}" uniqueName="18" name="Exclude Prohibited Chars Check" dataDxfId="117"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0400-000019000000}" uniqueName="stringRegEx" name="Regex" dataDxfId="116">
       <xmlColumnPr mapId="191" xpath="/root/datatype/stringRegEx" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" uniqueName="numMinVal" name="Min Value" dataDxfId="101">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" uniqueName="numMinVal" name="Min Value" dataDxfId="115">
       <xmlColumnPr mapId="191" xpath="/root/datatype/numMinVal" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0400-00000A000000}" uniqueName="numMaxVal" name="Max Value" dataDxfId="100">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0400-00000A000000}" uniqueName="numMaxVal" name="Max Value" dataDxfId="114">
       <xmlColumnPr mapId="191" xpath="/root/datatype/numMaxVal" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0400-00000C000000}" uniqueName="numDigitInteger" name="Integer Digits" dataDxfId="99">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0400-00000C000000}" uniqueName="numDigitInteger" name="Integer Digits" dataDxfId="113">
       <xmlColumnPr mapId="191" xpath="/root/datatype/numDigitInteger" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0400-00000D000000}" uniqueName="numDigitFraction" name="Decimal Digits" dataDxfId="98">
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0400-00000D000000}" uniqueName="numDigitFraction" name="Decimal Digits" dataDxfId="112">
       <xmlColumnPr mapId="191" xpath="/root/datatype/numDigitFraction" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" uniqueName="enumCodeLength" name="Code Length" dataDxfId="97">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" uniqueName="enumCodeLength" name="Code Length" dataDxfId="111">
       <xmlColumnPr mapId="191" xpath="/root/datatype/enumCodeLength" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0400-00000E000000}" uniqueName="notNeedsTimezone" name="No Timezone" dataDxfId="96">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0400-00000E000000}" uniqueName="notNeedsTimezone" name="No Timezone" dataDxfId="110">
       <xmlColumnPr mapId="191" xpath="/root/datatype/notNeedsTimezone" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{B168B020-1AF0-9B42-BEEA-270E7FD756C0}" uniqueName="6" name="Max Size [MB]"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0400-000010000000}" uniqueName="javadoc" name="Notes" dataDxfId="95">
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0400-000010000000}" uniqueName="javadoc" name="Notes" dataDxfId="109">
       <xmlColumnPr mapId="191" xpath="/root/datatype/javadoc" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" uniqueName="2" name="Pattern Desc (Default Lang)" dataDxfId="94"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0400-000013000000}" uniqueName="19" name="Pattern Desc (Additional Lang 1)" dataDxfId="93"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0400-000014000000}" uniqueName="20" name="Pattern Desc (Additional Lang 2)" dataDxfId="92"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0400-000015000000}" uniqueName="21" name="Pattern Desc (Additional Lang 3)" dataDxfId="91"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" uniqueName="2" name="Pattern Desc (Default Lang)" dataDxfId="108"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0400-000013000000}" uniqueName="19" name="Pattern Desc (Additional Lang 1)" dataDxfId="107"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0400-000014000000}" uniqueName="20" name="Pattern Desc (Additional Lang 2)" dataDxfId="106"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0400-000015000000}" uniqueName="21" name="Pattern Desc (Additional Lang 3)" dataDxfId="105"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Table4" displayName="Table4" ref="A6:I9" tableType="xml" totalsRowShown="0" headerRowDxfId="90" dataDxfId="89">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Table4" displayName="Table4" ref="A6:I9" tableType="xml" totalsRowShown="0" headerRowDxfId="89" dataDxfId="88">
   <autoFilter ref="A6:I9" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" uniqueName="dataTypeName" name="DataType Name" dataDxfId="88">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" uniqueName="dataTypeName" name="DataType Name" dataDxfId="87">
       <xmlColumnPr mapId="132" xpath="/root/enum/dataTypeName" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" uniqueName="8" name="code" dataDxfId="87"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" uniqueName="varName" name="varName" dataDxfId="86">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" uniqueName="8" name="code" dataDxfId="86"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" uniqueName="varName" name="varName" dataDxfId="85">
       <xmlColumnPr mapId="132" xpath="/root/enum/varName" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0500-00000A000000}" uniqueName="10" name="Java Only" dataDxfId="85"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0500-00000C000000}" uniqueName="javadoc-value" name="Notes" dataDxfId="84">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0500-00000A000000}" uniqueName="10" name="Java Only" dataDxfId="84"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0500-00000C000000}" uniqueName="javadoc-value" name="Notes" dataDxfId="83">
       <xmlColumnPr mapId="132" xpath="/root/enum/javadoc-value" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" uniqueName="9" name="Display Name (Default Lang)" dataDxfId="83"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" uniqueName="dispNameAddLang1" name="Display Name (Additional Lang 1)" dataDxfId="82">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" uniqueName="9" name="Display Name (Default Lang)" dataDxfId="82"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" uniqueName="dispNameAddLang1" name="Display Name (Additional Lang 1)" dataDxfId="81">
       <xmlColumnPr mapId="132" xpath="/root/enum/dispNameAddLang1" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" uniqueName="dispNameAddLang2" name="Display Name (Additional Lang 2)" dataDxfId="81">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" uniqueName="dispNameAddLang2" name="Display Name (Additional Lang 2)" dataDxfId="80">
       <xmlColumnPr mapId="132" xpath="/root/enum/dispNameAddLang2" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" uniqueName="dispNameAddLang3" name="Display Name (Additional Lang 3)" dataDxfId="80">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" uniqueName="dispNameAddLang3" name="Display Name (Additional Lang 3)" dataDxfId="79">
       <xmlColumnPr mapId="132" xpath="/root/enum/dispNameAddLang3" xmlDataType="string"/>
     </tableColumn>
   </tableColumns>
@@ -3126,83 +3129,83 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="Table7" displayName="Table7" ref="A5:AL8" tableType="xml" totalsRowShown="0" headerRowDxfId="79" dataDxfId="78">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="Table7" displayName="Table7" ref="A5:AL8" tableType="xml" totalsRowShown="0" headerRowDxfId="78" dataDxfId="77">
   <autoFilter ref="A5:AL8" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
   <tableColumns count="38">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" uniqueName="table" name="Table Name" dataDxfId="77">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" uniqueName="table" name="Table Name" dataDxfId="76">
       <xmlColumnPr mapId="161" xpath="/root/column/table" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" uniqueName="name" name="Column Name" dataDxfId="76">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" uniqueName="name" name="Column Name" dataDxfId="75">
       <xmlColumnPr mapId="161" xpath="/root/column/@name" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0600-00000F000000}" uniqueName="dataType" name="dataType" dataDxfId="75">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0600-00000F000000}" uniqueName="dataType" name="dataType" dataDxfId="74">
       <xmlColumnPr mapId="161" xpath="/root/column/dataType" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0600-000010000000}" uniqueName="16" name="dataType Check" dataDxfId="74">
-      <calculatedColumnFormula>IF(Table7[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table7[[#This Row],[dataType]], 'dataType Definition'!A:A, 1,FALSE))), "○", "×"))</calculatedColumnFormula>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0600-000010000000}" uniqueName="16" name="dataType Check" dataDxfId="73">
+      <calculatedColumnFormula>IF(Table7[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table7[[#This Row],[dataType]], 'DataType Definition'!A:A, 1,FALSE))), "○", "×"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0600-00001C000000}" uniqueName="28" name="Java Only" dataDxfId="73"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" uniqueName="pk" name="Surrogate key " dataDxfId="72">
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0600-00001C000000}" uniqueName="28" name="Java Only" dataDxfId="72"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" uniqueName="pk" name="Surrogate key " dataDxfId="71">
       <xmlColumnPr mapId="161" xpath="/root/column/pk" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0600-00001D000000}" uniqueName="29" name="natural key (unique key)" dataDxfId="71"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0600-000008000000}" uniqueName="nullable" name="nullable" dataDxfId="70">
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0600-00001D000000}" uniqueName="29" name="natural key (unique key)" dataDxfId="70"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0600-000008000000}" uniqueName="nullable" name="nullable" dataDxfId="69">
       <xmlColumnPr mapId="161" xpath="/root/column/nullable" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0600-00000A000000}" uniqueName="autoIncrement" name="Auto Numbering" dataDxfId="69">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0600-00000A000000}" uniqueName="autoIncrement" name="Auto Numbering" dataDxfId="68">
       <xmlColumnPr mapId="161" xpath="/root/column/autoIncrement" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0600-000015000000}" uniqueName="forcedIncrement" name="Force Numbering" dataDxfId="68">
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0600-000015000000}" uniqueName="forcedIncrement" name="Force Numbering" dataDxfId="67">
       <xmlColumnPr mapId="161" xpath="/root/column/forcedIncrement" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0600-00000B000000}" uniqueName="autoUpdate" name="Auto Update" dataDxfId="67">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0600-00000B000000}" uniqueName="autoUpdate" name="Auto Update" dataDxfId="66">
       <xmlColumnPr mapId="161" xpath="/root/column/autoUpdate" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0600-000014000000}" uniqueName="forcedUpdate" name="Force Update" dataDxfId="66">
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0600-000014000000}" uniqueName="forcedUpdate" name="Force Update" dataDxfId="65">
       <xmlColumnPr mapId="161" xpath="/root/column/forcedUpdate" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0600-00000C000000}" uniqueName="valueChangeMethod" name="Group Identifier" dataDxfId="65">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0600-00000C000000}" uniqueName="valueChangeMethod" name="Group Identifier" dataDxfId="64">
       <xmlColumnPr mapId="161" xpath="/root/column/valueChangeMethod" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0600-000012000000}" uniqueName="updatedValue" name="Spring Audit" dataDxfId="64">
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0600-000012000000}" uniqueName="updatedValue" name="Spring Audit" dataDxfId="63">
       <xmlColumnPr mapId="161" xpath="/root/column/updatedValue" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0600-000013000000}" uniqueName="optLock" name="Relation: Type" dataDxfId="63">
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0600-000013000000}" uniqueName="optLock" name="Relation: Type" dataDxfId="62">
       <xmlColumnPr mapId="161" xpath="/root/column/optLock" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0600-000016000000}" uniqueName="22" name="Relation: Direction" dataDxfId="62"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0600-00001A000000}" uniqueName="26" name="Relation: Source Var Name" dataDxfId="61"/>
-    <tableColumn id="31" xr3:uid="{9D7281DD-5315-4241-A8BB-439EC0CF8E4B}" uniqueName="31" name="Relation: Source Var itemNameKeyClass" dataDxfId="60"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0600-000017000000}" uniqueName="23" name="Relation: Target Table" dataDxfId="59"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0600-000018000000}" uniqueName="24" name="Relation: Target Column" dataDxfId="58"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0600-00001B000000}" uniqueName="27" name="Relation: Target Var Name" dataDxfId="57"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0600-000016000000}" uniqueName="22" name="Relation: Direction" dataDxfId="61"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0600-00001A000000}" uniqueName="26" name="Relation: Source Var Name" dataDxfId="60"/>
+    <tableColumn id="31" xr3:uid="{9D7281DD-5315-4241-A8BB-439EC0CF8E4B}" uniqueName="31" name="Relation: Source Var itemNameKeyClass" dataDxfId="59"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0600-000017000000}" uniqueName="23" name="Relation: Target Table" dataDxfId="58"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0600-000018000000}" uniqueName="24" name="Relation: Target Column" dataDxfId="57"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0600-00001B000000}" uniqueName="27" name="Relation: Target Var Name" dataDxfId="56"/>
     <tableColumn id="30" xr3:uid="{6428A7A6-FE3D-A242-BAE9-10F0BE9F39E9}" uniqueName="30" name="Relation: Target Var itemNameKeyClass"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0600-000019000000}" uniqueName="25" name="Relation: Eager" dataDxfId="56"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0600-000011000000}" uniqueName="index1" name="index1" dataDxfId="55">
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0600-000019000000}" uniqueName="25" name="Relation: Eager" dataDxfId="55"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0600-000011000000}" uniqueName="index1" name="index1" dataDxfId="54">
       <xmlColumnPr mapId="161" xpath="/root/column/index1" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0600-00000E000000}" uniqueName="index2" name="index2" dataDxfId="54">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0600-00000E000000}" uniqueName="index2" name="index2" dataDxfId="53">
       <xmlColumnPr mapId="161" xpath="/root/column/index2" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0600-00000D000000}" uniqueName="index3" name="index3" dataDxfId="53">
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0600-00000D000000}" uniqueName="index3" name="index3" dataDxfId="52">
       <xmlColumnPr mapId="161" xpath="/root/column/index3" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0600-000022000000}" uniqueName="34" name="index4" dataDxfId="52"/>
-    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0600-000023000000}" uniqueName="35" name="index5" dataDxfId="51"/>
-    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0600-000024000000}" uniqueName="36" name="index6" dataDxfId="50"/>
-    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0600-000025000000}" uniqueName="37" name="index7" dataDxfId="49"/>
-    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0600-000026000000}" uniqueName="38" name="index8" dataDxfId="48"/>
-    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0600-000027000000}" uniqueName="39" name="index9" dataDxfId="47"/>
-    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0600-000028000000}" uniqueName="40" name="index10" dataDxfId="46"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" uniqueName="dispNameAddLang1" name="Notes" dataDxfId="45"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0600-000009000000}" uniqueName="9" name="Column Display Name (Default Lang)" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" uniqueName="dispNameAddLang1" name="Column Display Name (Additional Lang 1)" dataDxfId="43">
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0600-000022000000}" uniqueName="34" name="index4" dataDxfId="51"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0600-000023000000}" uniqueName="35" name="index5" dataDxfId="50"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0600-000024000000}" uniqueName="36" name="index6" dataDxfId="49"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0600-000025000000}" uniqueName="37" name="index7" dataDxfId="48"/>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0600-000026000000}" uniqueName="38" name="index8" dataDxfId="47"/>
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0600-000027000000}" uniqueName="39" name="index9" dataDxfId="46"/>
+    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0600-000028000000}" uniqueName="40" name="index10" dataDxfId="45"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" uniqueName="dispNameAddLang1" name="Notes" dataDxfId="44"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0600-000009000000}" uniqueName="9" name="Column Display Name (Default Lang)" dataDxfId="43"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" uniqueName="dispNameAddLang1" name="Column Display Name (Additional Lang 1)" dataDxfId="42">
       <xmlColumnPr mapId="161" xpath="/root/column/dispNameAddLang1" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" uniqueName="dispNameAddLang2" name="Column Display Name (Additional Lang 2)" dataDxfId="42">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" uniqueName="dispNameAddLang2" name="Column Display Name (Additional Lang 2)" dataDxfId="41">
       <xmlColumnPr mapId="161" xpath="/root/column/dispNameAddLang2" xmlDataType="string"/>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" uniqueName="dispNameAddLang3" name="Column Display Name (Additional Lang 3)" dataDxfId="41">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" uniqueName="dispNameAddLang3" name="Column Display Name (Additional Lang 3)" dataDxfId="40">
       <xmlColumnPr mapId="161" xpath="/root/column/dispNameAddLang3" xmlDataType="string"/>
     </tableColumn>
   </tableColumns>
@@ -3211,49 +3214,49 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="Table74" displayName="Table74" ref="A5:AL8" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="Table74" displayName="Table74" ref="A5:AL8" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
   <autoFilter ref="A5:AL8" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="38">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="Table Name" dataDxfId="38"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Column Name" dataDxfId="37"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0700-00000F000000}" name="dataType" dataDxfId="36"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0700-000010000000}" name="dataType Check" dataDxfId="35">
-      <calculatedColumnFormula>IF(Table74[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table74[[#This Row],[dataType]], 'dataType Definition'!A:A, 1,FALSE))), "○", "×"))</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="Table Name" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Column Name" dataDxfId="36"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0700-00000F000000}" name="dataType" dataDxfId="35"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0700-000010000000}" name="dataType Check" dataDxfId="34">
+      <calculatedColumnFormula>IF(Table74[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table74[[#This Row],[dataType]], 'DataType Definition'!A:A, 1,FALSE))), "○", "×"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0700-00001C000000}" name="Java Only" dataDxfId="34"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="Surrogate key " dataDxfId="33"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="natural key (unique key)" dataDxfId="32"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0700-00001D000000}" name="nullable" dataDxfId="31"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0700-00000A000000}" name="Auto Numbering" dataDxfId="30"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0700-000015000000}" name="Force Numbering" dataDxfId="29"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Auto Update" dataDxfId="28"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0700-000014000000}" name="Force Update" dataDxfId="27"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0700-00000C000000}" name="Group Identifier" dataDxfId="26"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0700-000012000000}" name="Spring Audit" dataDxfId="25"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0700-000013000000}" name="Relation: Type" dataDxfId="24"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0700-000016000000}" name="Relation: Direction" dataDxfId="23"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0700-00001A000000}" name="Relation: Source Var Name" dataDxfId="22"/>
-    <tableColumn id="30" xr3:uid="{A60AB7BF-DE8E-F545-9E18-323611A659C9}" name="Relation: Source Var itemNameKeyClass" dataDxfId="21"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0700-000017000000}" name="Relation: Target Table" dataDxfId="20"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0700-000018000000}" name="Relation: Target Column" dataDxfId="19"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0700-00001B000000}" name="Relation: Target Var Name" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{B755CD40-B685-4E43-B654-6640AFFFB562}" name="Relation: Target Var itemNameKeyClass" dataDxfId="17"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0700-000019000000}" name="Relation: Eager" dataDxfId="16"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0700-000011000000}" name="index1" dataDxfId="15"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0700-00000E000000}" name="index2" dataDxfId="14"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0700-00000D000000}" name="index3" dataDxfId="13"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0700-000021000000}" name="index4" dataDxfId="12"/>
-    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0700-000022000000}" name="index5" dataDxfId="11"/>
-    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0700-000023000000}" name="index6" dataDxfId="10"/>
-    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0700-000024000000}" name="index7" dataDxfId="9"/>
-    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0700-000025000000}" name="index8" dataDxfId="8"/>
-    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0700-000026000000}" name="index9" dataDxfId="7"/>
-    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0700-000027000000}" name="index10" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="Notes" dataDxfId="5"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0700-000020000000}" name="Column Display Name (Default Lang)" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Column Display Name (Additional Lang 1)" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Column Display Name (Additional Lang 2)" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0700-000007000000}" name="Column Display Name (Additional Lang 3)" dataDxfId="1"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0700-00001C000000}" name="Java Only" dataDxfId="33"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="Surrogate key " dataDxfId="32"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="natural key (unique key)" dataDxfId="31"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0700-00001D000000}" name="nullable" dataDxfId="30"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0700-00000A000000}" name="Auto Numbering" dataDxfId="29"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0700-000015000000}" name="Force Numbering" dataDxfId="28"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Auto Update" dataDxfId="27"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0700-000014000000}" name="Force Update" dataDxfId="26"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0700-00000C000000}" name="Group Identifier" dataDxfId="25"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0700-000012000000}" name="Spring Audit" dataDxfId="24"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0700-000013000000}" name="Relation: Type" dataDxfId="23"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0700-000016000000}" name="Relation: Direction" dataDxfId="22"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0700-00001A000000}" name="Relation: Source Var Name" dataDxfId="21"/>
+    <tableColumn id="30" xr3:uid="{A60AB7BF-DE8E-F545-9E18-323611A659C9}" name="Relation: Source Var itemNameKeyClass" dataDxfId="20"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0700-000017000000}" name="Relation: Target Table" dataDxfId="19"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0700-000018000000}" name="Relation: Target Column" dataDxfId="18"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0700-00001B000000}" name="Relation: Target Var Name" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{B755CD40-B685-4E43-B654-6640AFFFB562}" name="Relation: Target Var itemNameKeyClass" dataDxfId="16"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0700-000019000000}" name="Relation: Eager" dataDxfId="15"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0700-000011000000}" name="index1" dataDxfId="14"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0700-00000E000000}" name="index2" dataDxfId="13"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0700-00000D000000}" name="index3" dataDxfId="12"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0700-000021000000}" name="index4" dataDxfId="11"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0700-000022000000}" name="index5" dataDxfId="10"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0700-000023000000}" name="index6" dataDxfId="9"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0700-000024000000}" name="index7" dataDxfId="8"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0700-000025000000}" name="index8" dataDxfId="7"/>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0700-000026000000}" name="index9" dataDxfId="6"/>
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0700-000027000000}" name="index10" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="Notes" dataDxfId="4"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0700-000020000000}" name="Column Display Name (Default Lang)" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Column Display Name (Additional Lang 1)" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Column Display Name (Additional Lang 2)" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0700-000007000000}" name="Column Display Name (Additional Lang 3)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3555,11 +3558,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="108" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="103"/>
-      <c r="C1" s="104"/>
+      <c r="B1" s="109"/>
+      <c r="C1" s="110"/>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="100" t="s">
@@ -5353,7 +5356,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="7" t="s">
-        <v>41</v>
+        <v>219</v>
       </c>
       <c r="B1" s="3"/>
     </row>
@@ -5404,38 +5407,38 @@
       <c r="B5" s="28" t="s">
         <v>174</v>
       </c>
-      <c r="C5" s="107" t="s">
+      <c r="C5" s="106" t="s">
         <v>175</v>
       </c>
-      <c r="D5" s="108"/>
-      <c r="E5" s="108"/>
-      <c r="F5" s="108"/>
-      <c r="G5" s="108"/>
-      <c r="H5" s="108"/>
-      <c r="I5" s="105" t="s">
+      <c r="D5" s="107"/>
+      <c r="E5" s="107"/>
+      <c r="F5" s="107"/>
+      <c r="G5" s="107"/>
+      <c r="H5" s="107"/>
+      <c r="I5" s="104" t="s">
         <v>176</v>
       </c>
-      <c r="J5" s="106"/>
-      <c r="K5" s="106"/>
-      <c r="L5" s="106"/>
+      <c r="J5" s="105"/>
+      <c r="K5" s="105"/>
+      <c r="L5" s="105"/>
       <c r="M5" s="30" t="s">
         <v>177</v>
       </c>
       <c r="N5" s="48" t="s">
         <v>178</v>
       </c>
-      <c r="O5" s="109" t="s">
+      <c r="O5" s="102" t="s">
         <v>218</v>
       </c>
       <c r="P5" s="51" t="s">
         <v>36</v>
       </c>
-      <c r="Q5" s="107" t="s">
+      <c r="Q5" s="106" t="s">
         <v>175</v>
       </c>
-      <c r="R5" s="106"/>
-      <c r="S5" s="106"/>
-      <c r="T5" s="106"/>
+      <c r="R5" s="105"/>
+      <c r="S5" s="105"/>
+      <c r="T5" s="105"/>
     </row>
     <row r="6" spans="1:20">
       <c r="B6" s="20" t="s">
@@ -5477,7 +5480,7 @@
       <c r="N6" s="47" t="s">
         <v>179</v>
       </c>
-      <c r="O6" s="110" t="s">
+      <c r="O6" s="103" t="s">
         <v>121</v>
       </c>
       <c r="P6" s="21" t="s">
@@ -6004,7 +6007,7 @@
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
       <c r="D6" s="43" t="str">
-        <f>IF(Table7[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table7[[#This Row],[dataType]], 'dataType Definition'!A:A, 1,FALSE))), "○", "×"))</f>
+        <f>IF(Table7[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table7[[#This Row],[dataType]], 'DataType Definition'!A:A, 1,FALSE))), "○", "×"))</f>
         <v/>
       </c>
       <c r="E6" s="9"/>
@@ -6048,7 +6051,7 @@
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
       <c r="D7" s="43" t="str">
-        <f>IF(Table7[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table7[[#This Row],[dataType]], 'dataType Definition'!A:A, 1,FALSE))), "○", "×"))</f>
+        <f>IF(Table7[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table7[[#This Row],[dataType]], 'DataType Definition'!A:A, 1,FALSE))), "○", "×"))</f>
         <v/>
       </c>
       <c r="E7" s="9"/>
@@ -6092,7 +6095,7 @@
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
       <c r="D8" s="43" t="str">
-        <f>IF(Table7[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table7[[#This Row],[dataType]], 'dataType Definition'!A:A, 1,FALSE))), "○", "×"))</f>
+        <f>IF(Table7[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table7[[#This Row],[dataType]], 'DataType Definition'!A:A, 1,FALSE))), "○", "×"))</f>
         <v/>
       </c>
       <c r="E8" s="9"/>
@@ -6347,7 +6350,7 @@
       <c r="B6" s="67"/>
       <c r="C6" s="66"/>
       <c r="D6" s="101" t="str">
-        <f>IF(Table74[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table74[[#This Row],[dataType]], 'dataType Definition'!A:A, 1,FALSE))), "○", "×"))</f>
+        <f>IF(Table74[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table74[[#This Row],[dataType]], 'DataType Definition'!A:A, 1,FALSE))), "○", "×"))</f>
         <v/>
       </c>
       <c r="E6" s="68"/>
@@ -6390,7 +6393,7 @@
       <c r="B7" s="75"/>
       <c r="C7" s="74"/>
       <c r="D7" s="101" t="str">
-        <f>IF(Table74[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table74[[#This Row],[dataType]], 'dataType Definition'!A:A, 1,FALSE))), "○", "×"))</f>
+        <f>IF(Table74[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table74[[#This Row],[dataType]], 'DataType Definition'!A:A, 1,FALSE))), "○", "×"))</f>
         <v/>
       </c>
       <c r="E7" s="76"/>
@@ -6433,7 +6436,7 @@
       <c r="B8" s="67"/>
       <c r="C8" s="78"/>
       <c r="D8" s="101" t="str">
-        <f>IF(Table74[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table74[[#This Row],[dataType]], 'dataType Definition'!A:A, 1,FALSE))), "○", "×"))</f>
+        <f>IF(Table74[[#This Row],[dataType]]="","",IF(NOT(ISNA(VLOOKUP(Table74[[#This Row],[dataType]], 'DataType Definition'!A:A, 1,FALSE))), "○", "×"))</f>
         <v/>
       </c>
       <c r="E8" s="68"/>

</xml_diff>